<commit_message>
Ajoute le journal des incidents au dictionnaire de données
Premier incident documenté : retrait par la NOAA du dossier
products/solar-wind, détecté par le manifeste et corrigé en passant
sur les flux temps réel RTSW.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Synthèse" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Vérification CGU" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Journal des incidents" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="230">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -644,17 +645,87 @@
   </si>
   <si>
     <t xml:space="preserve">Le scraping de valeurs numériques brutes (Kp, flux, taches solaires) n'est pas interdit par les CGU, à condition de citer les sources d'origine. À éviter : graphiques, images, mise en page. Le robots.txt l'autorise pour un robot générique avec un délai de 5 secondes entre requêtes, mais refuse l'entraînement d'IA (ai-train=no) : pour un modèle de ML, prendre NOAA et GFZ à la source ou demander l'accord du site. Bonnes pratiques : une collecte par heure, 5 secondes entre pages, User-Agent identifiable. Pages lues via un outil de résumé : relire les textes sur le site avant de les citer. Vérification faite le 26/10/2026, ce n'est pas un avis juridique.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Journal des incidents de collecte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un incident par ligne, du plus récent au plus ancien (C4.4.2 résolution d'incident, C1.1.2 exhaustivité de la collecte, C4.3.1 supervision).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N°</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date de détection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source / composant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Symptôme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment il a été détecté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cause</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date de résolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prévention / leçon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compétences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INC-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC : vent solaire (champ magnétique et plasma)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premier lancement de la collecte horaire (GitHub Actions) : 7 sources sur 9 collectées, les 2 sources du vent solaire en erreur HTTP 404.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manifeste de l'exécution (ok = false, http_status = 404) et exécution GitHub Actions marquée en échec par l'étape « Signaler un échec partiel ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La NOAA a retiré l'ancien dossier /products/solar-wind/ (mag-*.json, plasma-*.json). Les données sont désormais publiées dans /json/rtsw/ (rtsw_mag_1m.json, rtsw_wind_1m.json).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bz, Bt, vitesse et densité du vent solaire (variables essentielles) non collectés pendant ce lancement. Pas de perte durable : la collecte venait de démarrer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bascule sur les flux temps réel RTSW. Ces fichiers (1,4 à 2,4 Mo) sont réduits aux 3 dernières heures, sans modifier les enregistrements gardés ; le manifeste note les lignes reçues et gardées. Un flux figé (aucune donnée récente) est signalé en échec. Tests ajoutés. Commit d5bcc17.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correctif déployé, à confirmer au prochain lancement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lire le manifeste après chaque exécution. Vérifier les URL dans la documentation NOAA : le listing du répertoire affichait encore les anciens fichiers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4.4.2, C1.1.2, C4.3.1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -717,6 +788,13 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -785,7 +863,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -858,12 +936,24 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2361,7 +2451,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
         <v>205</v>
       </c>
@@ -2387,4 +2477,123 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="20" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="L4" s="17" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="B5" s="22" t="n">
+        <v>46321</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>46321</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>229</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Clôt l'incident INC-001 après vérification de la collecte
L'exécution #2 du 26/10/2026 collecte les 9 sources, vent solaire compris.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -704,10 +704,10 @@
     <t xml:space="preserve">Bz, Bt, vitesse et densité du vent solaire (variables essentielles) non collectés pendant ce lancement. Pas de perte durable : la collecte venait de démarrer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bascule sur les flux temps réel RTSW. Ces fichiers (1,4 à 2,4 Mo) sont réduits aux 3 dernières heures, sans modifier les enregistrements gardés ; le manifeste note les lignes reçues et gardées. Un flux figé (aucune donnée récente) est signalé en échec. Tests ajoutés. Commit d5bcc17.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correctif déployé, à confirmer au prochain lancement</t>
+    <t xml:space="preserve">Bascule sur les flux temps réel RTSW. Ces fichiers (1,4 à 2,4 Mo) sont réduits aux 3 dernières heures, sans modifier les enregistrements gardés ; le manifeste note les lignes reçues et gardées. Un flux figé (aucune donnée récente) est signalé en échec. Tests ajoutés. Commit d5bcc17. Vérifié le 26/10/2026 à 19:52 UTC (exécution #2) : 9 sources sur 9 collectées, 264 et 248 mesures de vent solaire gardées.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résolu</t>
   </si>
   <si>
     <t xml:space="preserve">Lire le manifeste après chaque exécution. Vérifier les URL dans la documentation NOAA : le listing du répertoire affichait encore les anciens fichiers.</t>
@@ -863,7 +863,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -944,11 +944,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2487,27 +2483,27 @@
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
         <v>208</v>
       </c>
     </row>
@@ -2549,11 +2545,11 @@
         <v>219</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="C5" s="16" t="s">
@@ -2574,7 +2570,7 @@
       <c r="H5" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="J5" s="16" t="s">

</xml_diff>

<commit_message>
Ajoute le backfill de l'historique du Kp depuis le GFZ
Télécharge le fichier Kp_ap_Ap_SN_F107 depuis 1932, l'archive tel quel et
produit un rapport de qualité (jours manquants ou en double, Kp hors
bornes, valeurs encore provisoires). Workflow manuel qui archive dans la
branche raw-data. Le dictionnaire de données pointe désormais vers les flux
temps réel RTSW du vent solaire et la licence GFZ est confirmée.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -89,7 +89,7 @@
     <t xml:space="preserve">Toutes les 3 h (relevé horaire avec dédoublonnage)</t>
   </si>
   <si>
-    <t xml:space="preserve">NOAA SWPC (JSON) ; historique GFZ / OMNIWeb (à vérifier)</t>
+    <t xml:space="preserve">NOAA SWPC (JSON) ; historique : GFZ Potsdam (Kp_ap_Ap_SN_F107_since_1932.txt)</t>
   </si>
   <si>
     <t xml:space="preserve">API</t>
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Mesure principale d'activité ; variable cible ou référence</t>
   </si>
   <si>
-    <t xml:space="preserve">NOAA : données publiques (à citer) ; GFZ : à vérifier</t>
+    <t xml:space="preserve">NOAA : données publiques (à citer) ; GFZ : CC BY 4.0 (taches solaires : CC BY-NC 4.0)</t>
   </si>
   <si>
     <t xml:space="preserve">À faire</t>
@@ -149,7 +149,7 @@
     <t xml:space="preserve">1 fois par heure : moyenne et minimum</t>
   </si>
   <si>
-    <t xml:space="preserve">NOAA SWPC (JSON, mag-7-day)</t>
+    <t xml:space="preserve">NOAA SWPC (JSON temps réel RTSW, /json/rtsw/rtsw_mag_1m.json)</t>
   </si>
   <si>
     <t xml:space="preserve">Court terme (30 à 60 min)</t>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">1 fois par heure : moyenne et maximum</t>
   </si>
   <si>
-    <t xml:space="preserve">NOAA SWPC (JSON, plasma-7-day)</t>
+    <t xml:space="preserve">NOAA SWPC (JSON temps réel RTSW, /json/rtsw/rtsw_wind_1m.json)</t>
   </si>
   <si>
     <t xml:space="preserve">Plus le vent est rapide, plus l'effet est fort</t>

</xml_diff>

<commit_message>
Respecte le robots.txt et ajoute les backfills OMNIWeb et Open-Meteo
Session HTTP partagée qui lit le robots.txt de chaque site avant de
télécharger (RFC 9309), respecte le Crawl-delay et note le résultat dans
le manifeste. Crawler du répertoire OMNIWeb pour le vent solaire horaire
et backfill de la nébulosité Open-Meteo par lieu et par année, chacun
avec son rapport de qualité. Un seul workflow de backfill au choix de la
source. Vérification des conditions d'utilisation des quatre sources
ajoutée au dictionnaire de données.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Synthèse" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Vérification CGU" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Journal des incidents" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Vérification CGU sources" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Journal des incidents" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="286">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -645,6 +646,174 @@
   </si>
   <si>
     <t xml:space="preserve">Le scraping de valeurs numériques brutes (Kp, flux, taches solaires) n'est pas interdit par les CGU, à condition de citer les sources d'origine. À éviter : graphiques, images, mise en page. Le robots.txt l'autorise pour un robot générique avec un délai de 5 secondes entre requêtes, mais refuse l'entraînement d'IA (ai-train=no) : pour un modèle de ML, prendre NOAA et GFZ à la source ou demander l'accord du site. Bonnes pratiques : une collecte par heure, 5 secondes entre pages, User-Agent identifiable. Pages lues via un outil de résumé : relire les textes sur le site avant de les citer. Vérification faite le 26/10/2026, ce n'est pas un avis juridique.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérification juridique : GFZ, NOAA SWPC, OMNIWeb (NASA), Open-Meteo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérification faite le 26/10/2026 (C1.1.2, cadre réglementaire). Ce n'est pas un avis juridique. Pages lues via un outil de résumé : relire les textes sur les sites avant de les citer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conséquence pour la collecte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GFZ Potsdam (Kp historique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page de l'indice Kp (GFZ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://gfz.de/en/section/geomagnetism/data-products-services/geomagnetic-kp-index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les données de l'indice Kp sont sous licence CC BY 4.0. Le GFZ demande d'être cité comme source des données.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citer le GFZ, le jeu de données (Matzka et al., 2021, Geomagnetic Kp index, GFZ Data Services, DOI 10.5880/Kp.0001) et l'article (Matzka et al., 2021, Space Weather, DOI 10.1029/2020SW002641).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En-tête du fichier Kp_ap_Ap_SN_F107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://kp.gfz.de/fileadmin/files_for_gfz_cms/Kp_ap_Ap_SN_F107_nowcast.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC BY 4.0, sauf le nombre de taches solaires (SN) : CC BY-NC 4.0, fourni par WDC-SILSO (Observatoire royal de Belgique). F10.7 fourni par le Dominion Radio Astrophysical Observatory et Ressources naturelles Canada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SN : usage non commercial seulement. Si AuroraCast devient un service payant, retirer SN ou demander l'accord de SILSO. Citer SILSO et DRAO / NRCan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page de téléchargement des données</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://kp.gfz.de/en/data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucune clause sur l'accès automatisé. La page conseille le téléchargement HTTPS pour les gros volumes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le backfill télécharge le fichier complet en HTTPS, une seule fois, à la demande.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC (collecte horaire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avertissement légal du NWS (dont dépend le SWPC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.weather.gov/DISCLAIMER.PHP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les informations des serveurs du gouvernement sont dans le domaine public, utilisables librement à condition de ne pas se les attribuer, de ne pas laisser croire à un soutien de la NOAA, et de ne pas présenter des données modifiées comme officielles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citer NOAA SWPC comme source. Dans l'application, présenter la prévision comme celle d'AuroraCast, jamais comme une prévision NOAA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiche data.gov « Space Weather Products »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://catalog-old.data.gov/dataset/space-weather-products2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Considéré comme une œuvre du gouvernement américain. Contraintes d'accès : aucune. Contraintes d'usage : aucune.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecte et réutilisation autorisées.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accès automatisé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://services.swpc.noaa.gov/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucune mention de limite de requêtes trouvée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonnes pratiques : une requête par heure et par fichier, User-Agent identifiable avec contact, nouvelles tentatives espacées.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMNIWeb (NASA SPDF, vent solaire historique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page « Citing OMNI »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://omniweb.gsfc.nasa.gov/html/citing.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citer le jeu de données OMNI horaire par son DOI en ajoutant la date d'accès ; remerciement suggéré : « We acknowledge use of NASA/GSFC's Space Physics Data Facility's OMNIWeb (or CDAWeb or ftp) service, and OMNI data ». Pas d'autre politique d'usage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citer Papitashvili et King (2020), OMNI Hourly Data, DOI 10.48322/1shr-ht18, avec la date d'accès, et King et Papitashvili (2005), DOI 10.1029/2004JA010649.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description du format omni2.text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://spdf.gsfc.nasa.gov/pub/data/omni/low_res_omni/omni2.text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les publications utilisant ces données doivent remercier le Space Physics Data Facility (SPDF).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mention du SPDF dans le dossier et la documentation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répertoire public des fichiers annuels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://spdf.gsfc.nasa.gov/pub/data/omni/low_res_omni/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répertoire public en HTTPS, un fichier par année (omni2_AAAA.dat, environ 2,7 Mo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crawling du répertoire pour découvrir les fichiers, puis téléchargement un par un avec une pause entre deux fichiers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open-Meteo (nébulosité historique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditions d'utilisation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open-meteo.com/en/terms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API gratuite réservée à l'usage non commercial (l'usage éducatif en fait partie ; les sites avec abonnement ou publicité sont commerciaux). Limites : moins de 10 000 appels par jour, 5 000 par heure, 600 par minute, 300 000 par mois.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet de certification : autorisé. Backfill découpé par lieu et par année, avec pause entre les appels. Si AuroraCast devient commercial : abonnement avec clé d'API.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open-meteo.com/en/licence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Données sous CC BY 4.0. Un lien « Weather data by Open-Meteo.com » doit figurer à côté de chaque endroit où les données sont affichées. Sources sous-jacentes listées, dont Copernicus (C3S) et l'ECMWF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afficher le lien Open-Meteo dans le tableau de bord du directeur ; citer Open-Meteo et Copernicus dans le dossier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toutes les sources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://kp.gfz.de/robots.txt ; https://services.swpc.noaa.gov/robots.txt ; https://spdf.gsfc.nasa.gov/robots.txt ; https://archive-api.open-meteo.com/robots.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non lisibles depuis l'outil de vérification le 26/10/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le collecteur lit le robots.txt de chaque site avant de télécharger, s'arrête si l'accès est interdit, respecte le Crawl-delay et note le résultat dans le manifeste.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les quatre sources autorisent la collecte et la réutilisation pour un projet de certification, à condition de les citer. Deux restrictions d'usage commercial sont à retenir : le nombre de taches solaires du fichier GFZ (CC BY-NC 4.0) et l'API gratuite d'Open-Meteo. Obligations d'affichage : le lien Open-Meteo à côté des données, et une prévision présentée comme celle d'AuroraCast, pas de la NOAA. Le respect du robots.txt est contrôlé automatiquement à chaque collecte.</t>
   </si>
   <si>
     <t xml:space="preserve">Journal des incidents de collecte</t>
@@ -863,7 +1032,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -942,6 +1111,18 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2480,6 +2661,280 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="20" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>246</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>254</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>255</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>258</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>259</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>260</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>262</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:E19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2499,88 +2954,88 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>207</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>208</v>
+      <c r="A2" s="23" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>209</v>
+        <v>265</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>210</v>
+        <v>266</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>211</v>
+        <v>267</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>212</v>
+        <v>268</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>213</v>
+        <v>269</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>214</v>
+        <v>270</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>215</v>
+        <v>271</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>216</v>
+        <v>272</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>217</v>
+        <v>273</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>218</v>
+        <v>274</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>219</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="B5" s="21" t="n">
+        <v>276</v>
+      </c>
+      <c r="B5" s="24" t="n">
         <v>46321</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>221</v>
+        <v>277</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>222</v>
+        <v>278</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>223</v>
+        <v>279</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>224</v>
+        <v>280</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>225</v>
+        <v>281</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>226</v>
-      </c>
-      <c r="I5" s="21" t="n">
+        <v>282</v>
+      </c>
+      <c r="I5" s="24" t="n">
         <v>46321</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>227</v>
+        <v>283</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>228</v>
+        <v>284</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>229</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remplace Open-Meteo par NOAA GHCNh et cherche les stations météo
Le robots.txt de l'API d'archive Open-Meteo interdit l'accès : la source
est retirée du backfill (incident INC-002). Ajout de la recherche des
stations GHCNh les plus proches des lieux cibles, avec examen d'un
fichier annuel pour vérifier que les nuages sont relevés. Journal des
incidents et vérification des conditions d'utilisation mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="307">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -648,7 +648,7 @@
     <t xml:space="preserve">Le scraping de valeurs numériques brutes (Kp, flux, taches solaires) n'est pas interdit par les CGU, à condition de citer les sources d'origine. À éviter : graphiques, images, mise en page. Le robots.txt l'autorise pour un robot générique avec un délai de 5 secondes entre requêtes, mais refuse l'entraînement d'IA (ai-train=no) : pour un modèle de ML, prendre NOAA et GFZ à la source ou demander l'accord du site. Bonnes pratiques : une collecte par heure, 5 secondes entre pages, User-Agent identifiable. Pages lues via un outil de résumé : relire les textes sur le site avant de les citer. Vérification faite le 26/10/2026, ce n'est pas un avis juridique.</t>
   </si>
   <si>
-    <t xml:space="preserve">Vérification juridique : GFZ, NOAA SWPC, OMNIWeb (NASA), Open-Meteo</t>
+    <t xml:space="preserve">Vérification juridique : GFZ, NOAA SWPC, OMNIWeb (NASA), Open-Meteo, NOAA GHCNh</t>
   </si>
   <si>
     <t xml:space="preserve">Vérification faite le 26/10/2026 (C1.1.2, cadre réglementaire). Ce n'est pas un avis juridique. Pages lues via un outil de résumé : relire les textes sur les sites avant de les citer.</t>
@@ -774,7 +774,7 @@
     <t xml:space="preserve">Crawling du répertoire pour découvrir les fichiers, puis téléchargement un par un avec une pause entre deux fichiers.</t>
   </si>
   <si>
-    <t xml:space="preserve">Open-Meteo (nébulosité historique)</t>
+    <t xml:space="preserve">Open-Meteo (nébulosité historique, écarté)</t>
   </si>
   <si>
     <t xml:space="preserve">Conditions d'utilisation</t>
@@ -801,19 +801,52 @@
     <t xml:space="preserve">Afficher le lien Open-Meteo dans le tableau de bord du directeur ; citer Open-Meteo et Copernicus dans le dossier.</t>
   </si>
   <si>
+    <t xml:space="preserve">NOAA GHCNh (nébulosité observée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiche data.gov GHCNh Version 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://catalog.data.gov/dataset/global-historical-climatology-network-hourly-ghcnh-version-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licence CC0 1.0 (domaine public). Remplace le jeu « Global Hourly » (ISD), qui n'est plus mis à jour depuis le 24/08/2025.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecte et réutilisation autorisées, y compris le stockage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registre AWS Open Data « NOAA GHCN-H »</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://registry.opendata.aws/noaa-ghcnh/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers publics dans l'espace noaa-ghcnh-pds (us-east-1). NOAA demande d'être citée pour un usage de données non modifiées et interdit de laisser croire à son soutien.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citer NOAA NCEI, GHCNh Version 1, DOI 10.25921/jp3d-3v19. Accès par fichier annuel par station, une requête par fichier avec pause.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA ISD Global Hourly (écarté)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avis NESDIS de changement de service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nesdis.noaa.gov/news/service-location-change-integrated-surface-data-global-hourly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produit remplacé : plus de mise à jour après le 24/08/2025 ; téléchargement direct retiré le 31/07/2026 ; GHCNh recommandé.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écarté : pas de données récentes.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Toutes les sources</t>
   </si>
   <si>
-    <t xml:space="preserve">https://kp.gfz.de/robots.txt ; https://services.swpc.noaa.gov/robots.txt ; https://spdf.gsfc.nasa.gov/robots.txt ; https://archive-api.open-meteo.com/robots.txt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non lisibles depuis l'outil de vérification le 26/10/2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le collecteur lit le robots.txt de chaque site avant de télécharger, s'arrête si l'accès est interdit, respecte le Crawl-delay et note le résultat dans le manifeste.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Les quatre sources autorisent la collecte et la réutilisation pour un projet de certification, à condition de les citer. Deux restrictions d'usage commercial sont à retenir : le nombre de taches solaires du fichier GFZ (CC BY-NC 4.0) et l'API gratuite d'Open-Meteo. Obligations d'affichage : le lien Open-Meteo à côté des données, et une prévision présentée comme celle d'AuroraCast, pas de la NOAA. Le respect du robots.txt est contrôlé automatiquement à chaque collecte.</t>
+    <t xml:space="preserve">GFZ, NOAA SWPC, OMNIWeb et NOAA GHCNh autorisent la collecte et la réutilisation pour un projet de certification, à condition de les citer. Open-Meteo est écarté : le robots.txt de son API d'archive interdit l'accès (incident INC-002). Restriction d'usage commercial à retenir : le nombre de taches solaires du fichier GFZ (CC BY-NC 4.0). Obligation d'affichage : une prévision présentée comme celle d'AuroraCast, pas de la NOAA. Le respect du robots.txt est contrôlé automatiquement à chaque collecte.</t>
   </si>
   <si>
     <t xml:space="preserve">Journal des incidents de collecte</t>
@@ -853,6 +886,36 @@
   </si>
   <si>
     <t xml:space="preserve">Compétences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INC-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open-Meteo : API d'archive (nébulosité historique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premier backfill : les 51 séries lieu-année Open-Meteo refusées, aucune donnée téléchargée (GFZ et OMNIWeb collectés sans erreur).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manifeste du backfill : robots = « lu », allowed = false, erreur « interdit par https://archive-api.open-meteo.com/robots.txt ». Exécution GitHub Actions en échec.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le robots.txt du sous-domaine archive-api.open-meteo.com interdit l'accès à tous les robots, alors que les conditions d'utilisation autorisent l'API gratuite en usage non commercial. Le contrôle robots.txt ajouté au collecteur a joué son rôle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pas d'historique de nébulosité. Sans effet sur le modèle de Kp (qui ne dépend pas du lieu) ; bloque l'analyse des nuits dégagées par lieu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Décision : appliquer strictement le robots.txt plutôt qu'une exception. Comparaison de sources (NASA POWER interdit par robots.txt ; NOAA ISD figé depuis le 24/08/2025) et choix de NOAA GHCNh (CC0, mis à jour chaque jour, accès autorisé). Open-Meteo retiré du workflow de backfill ; recherche des stations GHCNh proches des lieux cibles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contournement en cours : bascule vers NOAA GHCNh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrôler le robots.txt de chaque hôte (et pas seulement du site principal : open-meteo.com autorise, archive-api.open-meteo.com interdit) avant de retenir une source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1.1.2, C4.4.2, C3.3.3</t>
   </si>
   <si>
     <t xml:space="preserve">INC-001</t>
@@ -1032,7 +1095,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1111,18 +1174,6 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2661,27 +2712,27 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
         <v>8</v>
       </c>
@@ -2698,7 +2749,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
         <v>210</v>
       </c>
@@ -2715,7 +2766,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
         <v>210</v>
       </c>
@@ -2732,7 +2783,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
         <v>210</v>
       </c>
@@ -2749,7 +2800,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
         <v>223</v>
       </c>
@@ -2766,7 +2817,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
         <v>223</v>
       </c>
@@ -2783,7 +2834,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
         <v>223</v>
       </c>
@@ -2800,7 +2851,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
         <v>236</v>
       </c>
@@ -2817,7 +2868,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
         <v>236</v>
       </c>
@@ -2834,7 +2885,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
         <v>236</v>
       </c>
@@ -2851,7 +2902,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
         <v>249</v>
       </c>
@@ -2868,7 +2919,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
         <v>249</v>
       </c>
@@ -2885,40 +2936,79 @@
         <v>257</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
+    <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
         <v>258</v>
       </c>
-      <c r="B16" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="C16" s="16" t="s">
+      <c r="B16" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="C16" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="D16" s="1" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22" t="s">
+      <c r="E16" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>270</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>262</v>
-      </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
+    <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2935,7 +3025,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -2954,88 +3044,124 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
-        <v>264</v>
+      <c r="A2" s="20" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>269</v>
+        <v>280</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>272</v>
+        <v>283</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>276</v>
-      </c>
-      <c r="B5" s="24" t="n">
+        <v>287</v>
+      </c>
+      <c r="B5" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>282</v>
-      </c>
-      <c r="I5" s="24" t="n">
+        <v>293</v>
+      </c>
+      <c r="I5" s="21"/>
+      <c r="J5" s="16" t="s">
+        <v>294</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="B6" s="21" t="n">
         <v>46321</v>
       </c>
-      <c r="J5" s="16" t="s">
-        <v>283</v>
-      </c>
-      <c r="K5" s="16" t="s">
-        <v>284</v>
-      </c>
-      <c r="L5" s="16" t="s">
-        <v>285</v>
+      <c r="C6" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>300</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="K6" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="L6" s="16" t="s">
+        <v>306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Met à jour les statuts de collecte dans le dictionnaire de données
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="314">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -108,183 +108,198 @@
     <t xml:space="preserve">NOAA : données publiques (à citer) ; GFZ : CC BY 4.0 (taches solaires : CC BY-NC 4.0)</t>
   </si>
   <si>
+    <t xml:space="preserve">Collecté (NOAA toutes les heures ; historique GFZ depuis 1932)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kp prévu (3 jours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prévision NOAA du Kp, par tranche de 3 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 à 2 fois par jour ; conserver la date d'émission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC (JSON/texte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API + scraping du texte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moyen terme (1 à 3 jours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparer prévu vs observé (monitoring, bloc 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA : données publiques (à citer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté (NOAA toutes les heures, avec date d'émission)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bz (IMF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composante nord-sud du champ magnétique interplanétaire ; négatif = énergie qui entre dans la magnétosphère</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 fois par heure : moyenne et minimum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC (JSON temps réel RTSW, /json/rtsw/rtsw_mag_1m.json)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Court terme (30 à 60 min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meilleur indicateur d'une aurore imminente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté (NOAA RTSW toutes les heures ; historique OMNIWeb depuis 2010)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bt (IMF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intensité totale du champ magnétique interplanétaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 fois par heure : moyenne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Court terme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complète Bz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direction IMF (Bx, By)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orientation du champ interplanétaire ; le signe de Bz est ce qui compte le plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nT / degrés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 fois par heure (optionnel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optionnelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peu utile au début ; à tester en sélection de variables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté (NOAA RTSW ; By GSM dans OMNIWeb)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitesse du vent solaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitesse des particules du vent solaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">km/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 fois par heure : moyenne et maximum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC (JSON temps réel RTSW, /json/rtsw/rtsw_wind_1m.json)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plus le vent est rapide, plus l'effet est fort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Densité du vent solaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Densité de particules du vent solaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p/cm³</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amplifie l'effet de la vitesse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Échelle de tempête G1 à G5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niveau de tempête géomagnétique dérivé du Kp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niveau 0 à 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 fois par heure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC (JSON, noaa-scales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Étiquette lisible pour les agences et les alertes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté (NOAA toutes les heures)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alertes et avertissements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alertes, veilles et avertissements émis par NOAA (ex : Kp 5 attendu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Événementielle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toutes les heures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC (JSON, alerts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historiser les événements et déclencher des alertes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magnétomètre (brut)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mesures brutes des variations du champ magnétique (sol ou satellite)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non collecté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À déterminer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À écarter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redondant avec le Kp, qui en est dérivé</t>
+  </si>
+  <si>
     <t xml:space="preserve">À faire</t>
   </si>
   <si>
-    <t xml:space="preserve">Kp prévu (3 jours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prévision NOAA du Kp, par tranche de 3 h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 à 2 fois par jour ; conserver la date d'émission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOAA SWPC (JSON/texte)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API + scraping du texte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moyen terme (1 à 3 jours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comparer prévu vs observé (monitoring, bloc 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOAA : données publiques (à citer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bz (IMF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Composante nord-sud du champ magnétique interplanétaire ; négatif = énergie qui entre dans la magnétosphère</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 fois par heure : moyenne et minimum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOAA SWPC (JSON temps réel RTSW, /json/rtsw/rtsw_mag_1m.json)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Court terme (30 à 60 min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meilleur indicateur d'une aurore imminente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bt (IMF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intensité totale du champ magnétique interplanétaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 fois par heure : moyenne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Court terme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Utile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complète Bz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direction IMF (Bx, By)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orientation du champ interplanétaire ; le signe de Bz est ce qui compte le plus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nT / degrés</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 fois par heure (optionnel)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optionnelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peu utile au début ; à tester en sélection de variables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vitesse du vent solaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vitesse des particules du vent solaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">km/s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 fois par heure : moyenne et maximum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOAA SWPC (JSON temps réel RTSW, /json/rtsw/rtsw_wind_1m.json)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plus le vent est rapide, plus l'effet est fort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Densité du vent solaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Densité de particules du vent solaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p/cm³</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amplifie l'effet de la vitesse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Échelle de tempête G1 à G5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niveau de tempête géomagnétique dérivé du Kp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niveau 0 à 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 fois par heure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOAA SWPC (JSON, noaa-scales)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Étiquette lisible pour les agences et les alertes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alertes et avertissements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alertes, veilles et avertissements émis par NOAA (ex : Kp 5 attendu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Texte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Événementielle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toutes les heures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOAA SWPC (JSON, alerts)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Historiser les événements et déclencher des alertes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magnétomètre (brut)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mesures brutes des variations du champ magnétique (sol ou satellite)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non collecté</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À déterminer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À écarter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redondant avec le Kp, qui en est dérivé</t>
-  </si>
-  <si>
     <t xml:space="preserve">Phase de la Lune</t>
   </si>
   <si>
@@ -345,16 +360,19 @@
     <t xml:space="preserve">1 fois par jour (prévision + observé de la veille)</t>
   </si>
   <si>
-    <t xml:space="preserve">Open-Meteo (CSV / API archive) ; Frost MET Norway en complément</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API / CSV</t>
+    <t xml:space="preserve">NOAA GHCNh (stations TROMSO, aéroport de Kiruna, gare de Rovaniemi) ; Open-Meteo écarté (robots.txt, INC-002)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API (fichiers annuels)</t>
   </si>
   <si>
     <t xml:space="preserve">Un ciel couvert empêche de voir l'aurore</t>
   </si>
   <si>
-    <t xml:space="preserve">Open-Meteo : CC BY 4.0, non commercial ; Frost : NLOD 2.0 / CC 4.0</t>
+    <t xml:space="preserve">NOAA GHCNh : CC0 (citer NOAA NCEI, DOI 10.25921/jp3d-3v19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historique collecté (NOAA GHCNh 2010 → 24/10/2026) ; prévisions à faire</t>
   </si>
   <si>
     <t xml:space="preserve">Régions de taches solaires</t>
@@ -445,6 +463,9 @@
   </si>
   <si>
     <t xml:space="preserve">Illustre le scraping de données non structurées (C1.1.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté (NOAA toutes les heures), parsing à faire</t>
   </si>
   <si>
     <t xml:space="preserve">Synthèse des variables</t>
@@ -1607,235 +1628,235 @@
         <v>35</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J7" s="7" t="s">
         <v>24</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J10" s="7" t="s">
         <v>24</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J11" s="7" t="s">
         <v>24</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="L11" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>22</v>
@@ -1844,206 +1865,206 @@
         <v>23</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="L12" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="L13" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="E15" s="6" t="s">
+      <c r="J15" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="M15" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="G16" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>87</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>24</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="I17" s="7" t="s">
         <v>23</v>
@@ -2052,177 +2073,177 @@
         <v>24</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>27</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>33</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G19" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="H19" s="6" t="s">
-        <v>117</v>
-      </c>
       <c r="I19" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="L19" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="L21" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>27</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2276,7 +2297,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2284,7 +2305,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2298,7 +2319,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$21,A5)</f>
@@ -2307,7 +2328,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$21,A6)</f>
@@ -2316,7 +2337,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$21,A7)</f>
@@ -2325,7 +2346,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM(B4:B7)</f>
@@ -2334,7 +2355,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2348,7 +2369,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$21,"*"&amp;A12&amp;"*")</f>
@@ -2357,7 +2378,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$21,"*"&amp;A13&amp;"*")</f>
@@ -2389,71 +2410,71 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2484,209 +2505,209 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -2724,12 +2745,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2737,269 +2758,269 @@
         <v>8</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
@@ -3044,124 +3065,124 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="I5" s="21"/>
       <c r="J5" s="16" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="I6" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rend la collecte du vent solaire incrémentale et double les passages
L'ordonnanceur de GitHub n'a lancé que 2 passages en 13 heures (incident
INC-003). Chaque passage reprend désormais après la dernière mesure
archivée, lue dans les manifestes de la branche raw-data, avec 10 minutes
de recouvrement : un passage sauté ne fait plus perdre de mesures, et une
perte éventuelle est notée au manifeste. Deux passages par heure, à h17
et h47.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="324">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -907,6 +907,36 @@
   </si>
   <si>
     <t xml:space="preserve">Compétences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INC-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub Actions : planification de la collecte NOAA horaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entre le 26/10 à 19:52 UTC et le 27/10 à 08:40 UTC, seulement 2 passages automatiques (23:40 et 04:32 UTC, environ 33 min de retard) au lieu d'environ 13. Les deux passages ont collecté 9 sources sur 9.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparaison des commits horodatés de la branche raw-data avec la planification (cron « 7 * * * * »).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'ordonnanceur de GitHub Actions fonctionne au mieux : la documentation indique que les exécutions planifiées peuvent être retardées, voire supprimées, en période de forte charge, surtout aux heures pleines.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kp : aucune perte (le fichier NOAA couvre 7 jours). Vent solaire temps réel : environ 8 h de mesures perdues, à recompléter par OMNIWeb (publié avec environ un mois de retard). Prévisions et alertes émises entre deux passages : en partie perdues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecte incrémentale du vent solaire : chaque passage reprend après la dernière mesure archivée (lue dans les manifestes précédents), avec 10 min de recouvrement ; une perte n'est possible qu'au-delà de la profondeur du fichier NOAA (environ 2 jours) et elle est alors notée au manifeste (lost_from, lost_to). Deux passages par heure (h17 et h47), loin des heures pleines.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correctif déployé, à confirmer sur 24 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ne pas compter sur un ordonnanceur « au mieux » pour une collecte critique : argument pour Airflow (C1.1.3, C4.2.2). Concevoir les collectes pour être rattrapables (incrémentales et idempotentes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4.4.2, C1.1.3, C4.3.1</t>
   </si>
   <si>
     <t xml:space="preserve">INC-002</t>
@@ -3046,7 +3076,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -3116,7 +3146,7 @@
         <v>294</v>
       </c>
       <c r="B5" s="21" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>295</v>
@@ -3172,9 +3202,7 @@
       <c r="H6" s="16" t="s">
         <v>310</v>
       </c>
-      <c r="I6" s="21" t="n">
-        <v>46321</v>
-      </c>
+      <c r="I6" s="21"/>
       <c r="J6" s="16" t="s">
         <v>311</v>
       </c>
@@ -3183,6 +3211,44 @@
       </c>
       <c r="L6" s="16" t="s">
         <v>313</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>320</v>
+      </c>
+      <c r="I7" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>321</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dictionnaire : variables GSOD (SQL), licence GSOD/BigQuery, INC-004, INC-003 résolu, cadence 3 h
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="372">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -108,7 +108,7 @@
     <t xml:space="preserve">NOAA : données publiques (à citer) ; GFZ : CC BY 4.0 (taches solaires : CC BY-NC 4.0)</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecté (NOAA toutes les heures ; historique GFZ depuis 1932)</t>
+    <t xml:space="preserve">Collecté (NOAA toutes les 3 h ; historique GFZ depuis 1932)</t>
   </si>
   <si>
     <t xml:space="preserve">Kp prévu (3 jours)</t>
@@ -135,7 +135,7 @@
     <t xml:space="preserve">NOAA : données publiques (à citer)</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecté (NOAA toutes les heures, avec date d'émission)</t>
+    <t xml:space="preserve">Collecté (NOAA toutes les 3 h, avec date d'émission)</t>
   </si>
   <si>
     <t xml:space="preserve">Bz (IMF)</t>
@@ -150,7 +150,7 @@
     <t xml:space="preserve">Minute</t>
   </si>
   <si>
-    <t xml:space="preserve">1 fois par heure : moyenne et minimum</t>
+    <t xml:space="preserve">Toutes les 3 h (le flux garde environ 20 h) ; agrégé par heure : moyenne et minimum</t>
   </si>
   <si>
     <t xml:space="preserve">NOAA SWPC (JSON temps réel RTSW, /json/rtsw/rtsw_mag_1m.json)</t>
@@ -162,7 +162,7 @@
     <t xml:space="preserve">Meilleur indicateur d'une aurore imminente</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecté (NOAA RTSW toutes les heures ; historique OMNIWeb depuis 2010)</t>
+    <t xml:space="preserve">Collecté (NOAA RTSW toutes les 3 h ; historique OMNIWeb depuis 2010)</t>
   </si>
   <si>
     <t xml:space="preserve">Bt (IMF)</t>
@@ -243,7 +243,7 @@
     <t xml:space="preserve">Niveau 0 à 5</t>
   </si>
   <si>
-    <t xml:space="preserve">1 fois par heure</t>
+    <t xml:space="preserve">Toutes les 3 h</t>
   </si>
   <si>
     <t xml:space="preserve">NOAA SWPC (JSON, noaa-scales)</t>
@@ -252,7 +252,7 @@
     <t xml:space="preserve">Étiquette lisible pour les agences et les alertes</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecté (NOAA toutes les heures)</t>
+    <t xml:space="preserve">Collecté (NOAA toutes les 3 h)</t>
   </si>
   <si>
     <t xml:space="preserve">Alertes et avertissements</t>
@@ -267,7 +267,7 @@
     <t xml:space="preserve">Événementielle</t>
   </si>
   <si>
-    <t xml:space="preserve">Toutes les heures</t>
+    <t xml:space="preserve">Toutes les 3 h (le flux NOAA garde 30 jours)</t>
   </si>
   <si>
     <t xml:space="preserve">NOAA SWPC (JSON, alerts)</t>
@@ -465,7 +465,97 @@
     <t xml:space="preserve">Illustre le scraping de données non structurées (C1.1.2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecté (NOAA toutes les heures), parsing à faire</t>
+    <t xml:space="preserve">Collecté (NOAA toutes les 3 h), parsing à faire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Température (moyenne, min, max)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Température de l'air du jour, convertie de °F en °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">°C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historique : une fois (base figée au 24/08/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA NCEI GSOD, base publique BigQuery bigquery-public-data.noaa_gsod (stations TROMSO, KIRUNA, ROVANIEMI RAUTATIEASEMA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requêtes SQL (BigQuery)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contexte saisonnier ; froid sec souvent associé à un ciel dégagé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA NCEI : données publiques, sans garantie (citer « Global Surface Summary of the Day - GSOD », NCEI) ; requêtes BigQuery gratuites jusqu'à 1 To par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historique collecté et nettoyé (2010 → 24/08/2025, table weather_daily) ; prévisions à faire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point de rosée et humidité relative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point de rosée mesuré ; humidité relative calculée (formule de Magnus, à partir des moyennes du jour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">°C / %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historique : une fois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risque de brouillard et de givre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visibilité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visibilité horizontale moyenne du jour, convertie de miles en km</t>
+  </si>
+  <si>
+    <t xml:space="preserve">km</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brume et brouillard masquent le ciel comme les nuages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brouillard (jour signalé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vrai si la station a signalé du brouillard au moins une fois dans la journée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booléen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciel bouché en pleine saison des aurores (4 à 6 jours par mois en octobre-novembre à Kiruna et Rovaniemi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vent (moyen et maximum)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitesse moyenne et vitesse maximale soutenue du vent, converties de nœuds en m/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confort d'observation pour l'agence ; le vent dissipe aussi le brouillard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Précipitations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumul du jour, converti de pouces en mm ; lettre NOAA « I » (pas de relevé) passée à vide ; plus de 50 mm sans pluie signalée marqué suspect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exploitable seulement à Tromsø (92 % des jours) ; inutilisable à Kiruna et Rovaniemi (0 %)</t>
   </si>
   <si>
     <t xml:space="preserve">Synthèse des variables</t>
@@ -483,6 +573,9 @@
     <t xml:space="preserve">Scraping</t>
   </si>
   <si>
+    <t xml:space="preserve">SQL</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notes et points à vérifier</t>
   </si>
   <si>
@@ -507,7 +600,7 @@
     <t xml:space="preserve">Historique</t>
   </si>
   <si>
-    <t xml:space="preserve">Les JSON NOAA ne gardent que quelques jours. Prévoir un backfill (GFZ, OMNIWeb, Open-Meteo archive) puis une collecte continue.</t>
+    <t xml:space="preserve">Les JSON NOAA ne gardent que quelques heures à quelques jours (vent solaire environ 20 h, Kp observé 7 jours). Historique collecté une fois par backfill (GFZ depuis 1932, OMNIWeb, NOAA GHCNh et NOAA GSOD depuis 2010), puis collecte continue toutes les 3 h.</t>
   </si>
   <si>
     <t xml:space="preserve">Prévisions</t>
@@ -669,7 +762,7 @@
     <t xml:space="preserve">Le scraping de valeurs numériques brutes (Kp, flux, taches solaires) n'est pas interdit par les CGU, à condition de citer les sources d'origine. À éviter : graphiques, images, mise en page. Le robots.txt l'autorise pour un robot générique avec un délai de 5 secondes entre requêtes, mais refuse l'entraînement d'IA (ai-train=no) : pour un modèle de ML, prendre NOAA et GFZ à la source ou demander l'accord du site. Bonnes pratiques : une collecte par heure, 5 secondes entre pages, User-Agent identifiable. Pages lues via un outil de résumé : relire les textes sur le site avant de les citer. Vérification faite le 26/10/2026, ce n'est pas un avis juridique.</t>
   </si>
   <si>
-    <t xml:space="preserve">Vérification juridique : GFZ, NOAA SWPC, OMNIWeb (NASA), Open-Meteo, NOAA GHCNh</t>
+    <t xml:space="preserve">Vérification juridique : GFZ, NOAA SWPC, OMNIWeb (NASA), Open-Meteo, NOAA GHCNh, NOAA GSOD (BigQuery)</t>
   </si>
   <si>
     <t xml:space="preserve">Vérification faite le 26/10/2026 (C1.1.2, cadre réglementaire). Ce n'est pas un avis juridique. Pages lues via un outil de résumé : relire les textes sur les sites avant de les citer.</t>
@@ -864,10 +957,37 @@
     <t xml:space="preserve">Écarté : pas de données récentes.</t>
   </si>
   <si>
+    <t xml:space="preserve">NOAA GSOD (météo quotidienne, SQL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiche de métadonnées NCEI (GSOD, gov.noaa.ncdc:C00516)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ncei.noaa.gov/metadata/geoportal/rest/metadata/item/gov.noaa.ncdc:C00516/html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucune licence restrictive indiquée ; NOAA et NCEI ne donnent aucune garantie d'exactitude ou d'exhaustivité, l'utilisateur juge de l'usage des données. Citation demandée : « NOAA National Centers of Environmental Information. 1999. Global Surface Summary of the Day - GSOD. 1.0. [sous-ensemble utilisé]. Accessed [date] ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecte et réutilisation autorisées (œuvre du gouvernement américain, comme NOAA SWPC). Citer NCEI avec les 3 stations et la date d'accès. Qualité vérifiée par nos soins (rapport de qualité, incident INC-004).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google BigQuery, programme Public Datasets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://docs.cloud.google.com/bigquery/public-data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google paie le stockage ; l'utilisateur ne paie que ses requêtes, le premier To par mois est gratuit, et le mode sans facturation (sandbox) suffit en dessous. Pas de garantie de service (SLA). Les conditions propres aux données sont celles de leur producteur (ici la NOAA).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mode sandbox, sans carte bancaire. Chaque requête est d'abord estimée à blanc puis plafonnée à 15 Go (la plus grosse lit 8,7 Go). Compte de service limité au rôle « Utilisateur de job BigQuery ».</t>
+  </si>
+  <si>
     <t xml:space="preserve">Toutes les sources</t>
   </si>
   <si>
-    <t xml:space="preserve">GFZ, NOAA SWPC, OMNIWeb et NOAA GHCNh autorisent la collecte et la réutilisation pour un projet de certification, à condition de les citer. Open-Meteo est écarté : le robots.txt de son API d'archive interdit l'accès (incident INC-002). Restriction d'usage commercial à retenir : le nombre de taches solaires du fichier GFZ (CC BY-NC 4.0). Obligation d'affichage : une prévision présentée comme celle d'AuroraCast, pas de la NOAA. Le respect du robots.txt est contrôlé automatiquement à chaque collecte.</t>
+    <t xml:space="preserve">GFZ, NOAA SWPC, OMNIWeb, NOAA GHCNh et NOAA GSOD (via BigQuery) autorisent la collecte et la réutilisation pour un projet de certification, à condition de les citer. Open-Meteo est écarté : le robots.txt de son API d'archive interdit l'accès (incident INC-002). Restriction d'usage commercial à retenir : le nombre de taches solaires du fichier GFZ (CC BY-NC 4.0). Obligation d'affichage : une prévision présentée comme celle d'AuroraCast, pas de la NOAA. Coût BigQuery : nul tant que les requêtes restent sous 1 To par mois. Le respect du robots.txt est contrôlé automatiquement à chaque collecte.</t>
   </si>
   <si>
     <t xml:space="preserve">Journal des incidents de collecte</t>
@@ -909,6 +1029,36 @@
     <t xml:space="preserve">Compétences</t>
   </si>
   <si>
+    <t xml:space="preserve">INC-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google BigQuery : base existante bigquery-public-data.noaa_gsod (table stations)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backfill SQL GSOD en échec : pour les 3 lieux, « aucune station active à moins de 30 km », alors que les stations TROMSO (0,9 km), KIRUNA (6 km) et ROVANIEMI RAUTATIEASEMA (0,7 km) existent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lecture des résultats de la requête des stations archivés (stations_&lt;lieu&gt;.json) : la colonne « end » vaut 20210920 pour toutes les stations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La table de métadonnées « stations » n'est plus mise à jour depuis le 20/09/2021, alors que les tables annuelles de relevés vont jusqu'au 24/08/2025. Le collecteur jugeait l'activité d'une station sur cette date de fin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucune donnée météo quotidienne collectée pendant ce lancement. Pas de perte durable : la base est historique.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'activité d'une station est désormais mesurée dans les relevés eux-mêmes : la requête des stations est jointe (LEFT JOIN) aux relevés de la dernière année et compte les jours mesurés ; une station est retenue avec au moins 30 jours. Test ajouté (commit fd4ff50). Vérifié le 27/10/2026 à 10:45 UTC : 3 stations retenues (236 jours en 2025 chacune), 16 832 jours collectés pour 2010-2025, 8,7 Go lus, coût nul.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résolu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ne pas faire confiance aux métadonnées d'une base existante : contrôler dans les données elles-mêmes (qualité des données, C1.1.2). Archiver le résultat de chaque requête pour pouvoir diagnostiquer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1.1.2, C4.4.2</t>
+  </si>
+  <si>
     <t xml:space="preserve">INC-003</t>
   </si>
   <si>
@@ -927,13 +1077,10 @@
     <t xml:space="preserve">Kp : aucune perte (le fichier NOAA couvre 7 jours). Vent solaire temps réel : environ 8 h de mesures perdues, à recompléter par OMNIWeb (publié avec environ un mois de retard). Prévisions et alertes émises entre deux passages : en partie perdues.</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecte incrémentale du vent solaire : chaque passage reprend après la dernière mesure archivée (lue dans les manifestes précédents), avec 10 min de recouvrement ; une perte n'est possible qu'au-delà de la profondeur du fichier NOAA (environ 2 jours) et elle est alors notée au manifeste (lost_from, lost_to). Deux passages par heure (h17 et h47), loin des heures pleines.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correctif déployé, à confirmer sur 24 h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ne pas compter sur un ordonnanceur « au mieux » pour une collecte critique : argument pour Airflow (C1.1.3, C4.2.2). Concevoir les collectes pour être rattrapables (incrémentales et idempotentes).</t>
+    <t xml:space="preserve">Collecte incrémentale du vent solaire : chaque passage reprend après la dernière mesure archivée (lue dans les manifestes précédents), avec 10 min de recouvrement ; une perte n'est possible qu'au-delà de la profondeur du fichier NOAA (environ 20 h, mesurée sur les fichiers archivés) et elle est alors notée au manifeste (lost_from, lost_to). Vérifié du 27/10 au 29/10/2026 : GitHub n'a lancé la collecte que toutes les 4 à 6 h, sans aucune minute de vent solaire perdue. Cadence ensuite fixée à un passage toutes les 3 h (cron « 17 */3 * * * », commit 94f987f), choisie d'après la profondeur mesurée des flux : vent solaire environ 20 h, Kp observé 7 jours, alertes 30 jours ; seul kp_1m (environ 6 h) peut garder des trous, sans effet sur le modèle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ne pas compter sur un ordonnanceur « au mieux » pour une collecte critique : argument pour Airflow (C1.1.3, C4.2.2). Concevoir les collectes pour être rattrapables (incrémentales et idempotentes), et choisir la fréquence d'après la profondeur mesurée de chaque flux plutôt qu'au plus souvent possible.</t>
   </si>
   <si>
     <t xml:space="preserve">C4.4.2, C1.1.3, C4.3.1</t>
@@ -960,7 +1107,7 @@
     <t xml:space="preserve">Décision : appliquer strictement le robots.txt plutôt qu'une exception. Comparaison de sources (NASA POWER interdit par robots.txt ; NOAA ISD figé depuis le 24/08/2025) et choix de NOAA GHCNh (CC0, mis à jour chaque jour, accès autorisé). Open-Meteo retiré du workflow de backfill ; recherche des stations GHCNh proches des lieux cibles.</t>
   </si>
   <si>
-    <t xml:space="preserve">Contournement en cours : bascule vers NOAA GHCNh</t>
+    <t xml:space="preserve">Résolu (bascule vers NOAA GHCNh, historique collecté)</t>
   </si>
   <si>
     <t xml:space="preserve">Contrôler le robots.txt de chaque hôte (et pas seulement du site principal : open-meteo.com autorise, archive-api.open-meteo.com interdit) avant de retenir une source.</t>
@@ -988,9 +1135,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bascule sur les flux temps réel RTSW. Ces fichiers (1,4 à 2,4 Mo) sont réduits aux 3 dernières heures, sans modifier les enregistrements gardés ; le manifeste note les lignes reçues et gardées. Un flux figé (aucune donnée récente) est signalé en échec. Tests ajoutés. Commit d5bcc17. Vérifié le 26/10/2026 à 19:52 UTC (exécution #2) : 9 sources sur 9 collectées, 264 et 248 mesures de vent solaire gardées.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Résolu</t>
   </si>
   <si>
     <t xml:space="preserve">Lire le manifeste après chaque exécution. Vérifier les URL dans la documentation NOAA : le listing du répertoire affichait encore les anciens fichiers.</t>
@@ -1510,7 +1654,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -2170,7 +2314,7 @@
         <v>40</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>129</v>
@@ -2276,8 +2420,254 @@
         <v>146</v>
       </c>
     </row>
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J5:J21">
+  <conditionalFormatting sqref="J5:J27">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Essentielle"</formula>
     </cfRule>
@@ -2288,17 +2678,17 @@
       <formula>"À écarter"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M21">
+  <conditionalFormatting sqref="M5:M27">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminé"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M21" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M27" type="list">
       <formula1>"À faire,En cours,Terminé"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J21" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J27" type="list">
       <formula1>"Essentielle,Utile,Optionnelle,À écarter"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2318,7 +2708,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
@@ -2327,7 +2717,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>147</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2335,7 +2725,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2343,8 +2733,8 @@
         <v>24</v>
       </c>
       <c r="B4" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$21,A4)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A4)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2352,8 +2742,8 @@
         <v>50</v>
       </c>
       <c r="B5" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$21,A5)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A5)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2361,8 +2751,8 @@
         <v>56</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$21,A6)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A6)</f>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2370,22 +2760,22 @@
         <v>88</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$21,A7)</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A7)</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2393,16 +2783,16 @@
         <v>22</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$21,"*"&amp;A11&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A11&amp;"*")</f>
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$21,"*"&amp;A12&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A12&amp;"*")</f>
         <v>5</v>
       </c>
     </row>
@@ -2411,8 +2801,17 @@
         <v>98</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$21,"*"&amp;A13&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A13&amp;"*")</f>
         <v>2</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A14&amp;"*")</f>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2440,63 +2839,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>154</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>155</v>
+        <v>186</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>158</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>159</v>
+        <v>190</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>160</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>161</v>
+        <v>192</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>162</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>163</v>
+        <v>194</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>166</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2504,7 +2903,7 @@
         <v>137</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>167</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -2535,209 +2934,209 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>168</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>169</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>170</v>
+        <v>201</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>171</v>
+        <v>202</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>172</v>
+        <v>203</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>173</v>
+        <v>204</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>174</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>175</v>
+        <v>206</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>176</v>
+        <v>207</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>178</v>
+        <v>209</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>179</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>175</v>
+        <v>206</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>176</v>
+        <v>207</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>180</v>
+        <v>211</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>181</v>
+        <v>212</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>182</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>175</v>
+        <v>206</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>176</v>
+        <v>207</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>183</v>
+        <v>214</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>184</v>
+        <v>215</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>185</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>186</v>
+        <v>217</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>187</v>
+        <v>218</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>188</v>
+        <v>219</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>189</v>
+        <v>220</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>190</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>191</v>
+        <v>222</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>192</v>
+        <v>223</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>193</v>
+        <v>224</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>194</v>
+        <v>225</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>195</v>
+        <v>226</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>197</v>
+        <v>228</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>198</v>
+        <v>229</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>199</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>195</v>
+        <v>226</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>200</v>
+        <v>231</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>201</v>
+        <v>232</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>202</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>195</v>
+        <v>226</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>203</v>
+        <v>234</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>204</v>
+        <v>235</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>205</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>195</v>
+        <v>226</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>206</v>
+        <v>237</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>207</v>
+        <v>238</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>208</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>195</v>
+        <v>226</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>209</v>
+        <v>240</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>210</v>
+        <v>241</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>211</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>212</v>
+        <v>243</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>213</v>
+        <v>244</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -2763,7 +3162,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -2775,12 +3174,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>214</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>215</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2788,278 +3187,313 @@
         <v>8</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>170</v>
+        <v>201</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>171</v>
+        <v>202</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>173</v>
+        <v>204</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>216</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>217</v>
+        <v>248</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>218</v>
+        <v>249</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>219</v>
+        <v>250</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>220</v>
+        <v>251</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>221</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>217</v>
+        <v>248</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>222</v>
+        <v>253</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>223</v>
+        <v>254</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>224</v>
+        <v>255</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>225</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>217</v>
+        <v>248</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>226</v>
+        <v>257</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>227</v>
+        <v>258</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>228</v>
+        <v>259</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>229</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>230</v>
+        <v>261</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>231</v>
+        <v>262</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>232</v>
+        <v>263</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>233</v>
+        <v>264</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>234</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>230</v>
+        <v>261</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>235</v>
+        <v>266</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>236</v>
+        <v>267</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>237</v>
+        <v>268</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>238</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>230</v>
+        <v>261</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>239</v>
+        <v>270</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>240</v>
+        <v>271</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>241</v>
+        <v>272</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>242</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>243</v>
+        <v>274</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>244</v>
+        <v>275</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>245</v>
+        <v>276</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>246</v>
+        <v>277</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>247</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>243</v>
+        <v>274</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>248</v>
+        <v>279</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>249</v>
+        <v>280</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>250</v>
+        <v>281</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>251</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>243</v>
+        <v>274</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>252</v>
+        <v>283</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>253</v>
+        <v>284</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>254</v>
+        <v>285</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>255</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>256</v>
+        <v>287</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>257</v>
+        <v>288</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>258</v>
+        <v>289</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>259</v>
+        <v>290</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>260</v>
+        <v>291</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>256</v>
+        <v>287</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>261</v>
+        <v>292</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>262</v>
+        <v>293</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>263</v>
+        <v>294</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>264</v>
+        <v>295</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>267</v>
+        <v>298</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>268</v>
+        <v>299</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>269</v>
+        <v>300</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>270</v>
+        <v>301</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>271</v>
+        <v>302</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>272</v>
+        <v>303</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>273</v>
+        <v>304</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>274</v>
+        <v>305</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>275</v>
+        <v>306</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>276</v>
+        <v>307</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>279</v>
+        <v>310</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="s">
+        <v>310</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="E20" s="16" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>280</v>
-      </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
+      <c r="A21" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
+        <v>320</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A24:E24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3076,7 +3510,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -3095,160 +3529,200 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>281</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>282</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>283</v>
+        <v>323</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>284</v>
+        <v>324</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>285</v>
+        <v>325</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>286</v>
+        <v>326</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>287</v>
+        <v>327</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>288</v>
+        <v>328</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>289</v>
+        <v>329</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>290</v>
+        <v>330</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>291</v>
+        <v>331</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>292</v>
+        <v>332</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>294</v>
+        <v>334</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>295</v>
+        <v>335</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>296</v>
+        <v>336</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>297</v>
+        <v>337</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>298</v>
+        <v>338</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>299</v>
+        <v>339</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>300</v>
-      </c>
-      <c r="I5" s="21"/>
+        <v>340</v>
+      </c>
+      <c r="I5" s="21" t="n">
+        <v>46322</v>
+      </c>
       <c r="J5" s="16" t="s">
-        <v>301</v>
+        <v>341</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>302</v>
+        <v>342</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>303</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>304</v>
+        <v>344</v>
       </c>
       <c r="B6" s="21" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>305</v>
+        <v>345</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>306</v>
+        <v>346</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>307</v>
+        <v>347</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>308</v>
+        <v>348</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>309</v>
+        <v>349</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>310</v>
-      </c>
-      <c r="I6" s="21"/>
+        <v>350</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>46324</v>
+      </c>
       <c r="J6" s="16" t="s">
-        <v>311</v>
+        <v>341</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>312</v>
+        <v>351</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>314</v>
+        <v>353</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>315</v>
+        <v>354</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>316</v>
+        <v>355</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>317</v>
+        <v>356</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>318</v>
+        <v>357</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>319</v>
+        <v>358</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>320</v>
-      </c>
-      <c r="I7" s="21" t="n">
+        <v>359</v>
+      </c>
+      <c r="I7" s="21"/>
+      <c r="J7" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="B8" s="21" t="n">
         <v>46321</v>
       </c>
-      <c r="J7" s="16" t="s">
-        <v>321</v>
-      </c>
-      <c r="K7" s="16" t="s">
-        <v>322</v>
-      </c>
-      <c r="L7" s="16" t="s">
-        <v>323</v>
+      <c r="C8" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="I8" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Météo horaire GHCNh (weather_hourly), contrôle croisé avec GSOD, mise à jour quotidienne incrémentale de GHCNh
- transform/weather_hourly.py : température, humidité, pression, vent, visibilité, brouillard
  et brume par heure, 2010 -> hier ; codes qualité, vent 999, visibilité METAR plafonnée
- contrôle croisé : moyenne quotidienne recalculée contre GSOD (écart 0,03 à 0,09 °C)
- collect/ghcnh.py update + workflow quotidien : lignes nouvelles seulement (quelques Ko/jour)
- notebook 03 : contrôle croisé et relais GSOD -> GHCNh ; dictionnaire et README à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="386">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -477,7 +477,85 @@
     <t xml:space="preserve">°C</t>
   </si>
   <si>
-    <t xml:space="preserve">Historique : une fois (base figée au 24/08/2025)</t>
+    <t xml:space="preserve">Horaire (GHCNh) ; journalière (GSOD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GSOD : une fois (base figée) ; GHCNh : chaque jour, lignes nouvelles seulement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA NCEI GSOD par SQL (BigQuery bigquery-public-data.noaa_gsod, 2010 → 24/08/2025) ; NOAA GHCNh horaire, mêmes stations (TROMSO, aéroport de Kiruna, gare de Rovaniemi), 2010 → hier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requêtes SQL (BigQuery) + API (fichiers GHCNh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contexte saisonnier ; froid sec souvent associé à un ciel dégagé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA NCEI GSOD : données publiques, sans garantie (citer NCEI) ; NOAA GHCNh : CC0 (DOI 10.25921/jp3d-3v19) ; requêtes BigQuery gratuites jusqu'à 1 To par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté et nettoyé : GSOD (weather_daily) et GHCNh (weather_hourly, mis à jour chaque jour) ; contrôle croisé de la température : écart moyen 0,03 à 0,09 °C ; prévisions à faire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point de rosée et humidité relative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point de rosée mesuré ; humidité relative calculée (formule de Magnus, à partir des moyennes du jour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">°C / %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risque de brouillard et de givre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visibilité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visibilité horizontale, en km ; GSOD : moyenne du jour convertie des miles ; GHCNh : par heure. Messages METAR (aéroport de Kiruna) plafonnés à 10 km (« 10 km ou plus », colonne visibility_capped)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">km</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brume et brouillard masquent le ciel comme les nuages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brouillard (jour signalé)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brouillard signalé : GSOD = au moins une fois dans la journée ; GHCNh = par heure, d'après le temps présent WMO (abréviation FG, code manuel 40-49, automatique 30-35) ; brume (BR, code 10) en colonne séparée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booléen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciel bouché en pleine saison des aurores (4 à 6 jours par mois en octobre-novembre à Kiruna et Rovaniemi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vent (moyen et maximum)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vitesse (et direction pour GHCNh) du vent, en m/s ; direction 999 = vent calme ou variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confort d'observation pour l'agence ; le vent dissipe aussi le brouillard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Précipitations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumul du jour, converti de pouces en mm ; lettre NOAA « I » (pas de relevé) passée à vide ; plus de 50 mm sans pluie signalée marqué suspect</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historique : une fois</t>
   </si>
   <si>
     <t xml:space="preserve">NOAA NCEI GSOD, base publique BigQuery bigquery-public-data.noaa_gsod (stations TROMSO, KIRUNA, ROVANIEMI RAUTATIEASEMA)</t>
@@ -486,7 +564,7 @@
     <t xml:space="preserve">Requêtes SQL (BigQuery)</t>
   </si>
   <si>
-    <t xml:space="preserve">Contexte saisonnier ; froid sec souvent associé à un ciel dégagé</t>
+    <t xml:space="preserve">Exploitable seulement à Tromsø (92 % des jours) ; inutilisable à Kiruna et Rovaniemi (0 %)</t>
   </si>
   <si>
     <t xml:space="preserve">NOAA NCEI : données publiques, sans garantie (citer « Global Surface Summary of the Day - GSOD », NCEI) ; requêtes BigQuery gratuites jusqu'à 1 To par mois</t>
@@ -495,67 +573,31 @@
     <t xml:space="preserve">Historique collecté et nettoyé (2010 → 24/08/2025, table weather_daily) ; prévisions à faire</t>
   </si>
   <si>
-    <t xml:space="preserve">Point de rosée et humidité relative</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Point de rosée mesuré ; humidité relative calculée (formule de Magnus, à partir des moyennes du jour)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">°C / %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Historique : une fois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risque de brouillard et de givre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visibilité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visibilité horizontale moyenne du jour, convertie de miles en km</t>
-  </si>
-  <si>
-    <t xml:space="preserve">km</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brume et brouillard masquent le ciel comme les nuages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brouillard (jour signalé)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vrai si la station a signalé du brouillard au moins une fois dans la journée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Booléen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ciel bouché en pleine saison des aurores (4 à 6 jours par mois en octobre-novembre à Kiruna et Rovaniemi)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vent (moyen et maximum)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vitesse moyenne et vitesse maximale soutenue du vent, converties de nœuds en m/s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m/s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confort d'observation pour l'agence ; le vent dissipe aussi le brouillard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Précipitations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cumul du jour, converti de pouces en mm ; lettre NOAA « I » (pas de relevé) passée à vide ; plus de 50 mm sans pluie signalée marqué suspect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exploitable seulement à Tromsø (92 % des jours) ; inutilisable à Kiruna et Rovaniemi (0 %)</t>
+    <t xml:space="preserve">Pression au niveau de la mer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pression atmosphérique ramenée au niveau de la mer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hPa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chaque jour, lignes nouvelles seulement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA GHCNh horaire (TROMSO, aéroport de Kiruna, gare de Rovaniemi), 2010 → hier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API (fichiers GHCNh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Une pression qui monte annonce souvent un ciel qui se dégage ; à tester en sélection de variables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA GHCNh : CC0 (DOI 10.25921/jp3d-3v19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté et nettoyé (weather_hourly, 2010 → hier) ; prévisions à faire</t>
   </si>
   <si>
     <t xml:space="preserve">Synthèse des variables</t>
@@ -1654,7 +1696,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -2434,16 +2476,16 @@
         <v>149</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>23</v>
@@ -2452,39 +2494,39 @@
         <v>50</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>106</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>49</v>
@@ -2496,10 +2538,10 @@
         <v>160</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2516,16 +2558,16 @@
         <v>163</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I24" s="7" t="s">
         <v>49</v>
@@ -2537,10 +2579,10 @@
         <v>164</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M24" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2557,16 +2599,16 @@
         <v>167</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>49</v>
@@ -2578,10 +2620,10 @@
         <v>168</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2598,16 +2640,16 @@
         <v>171</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>49</v>
@@ -2619,10 +2661,10 @@
         <v>172</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2642,13 +2684,13 @@
         <v>120</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>151</v>
+        <v>177</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>49</v>
@@ -2657,17 +2699,58 @@
         <v>56</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>155</v>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J5:J27">
+  <conditionalFormatting sqref="J5:J28">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Essentielle"</formula>
     </cfRule>
@@ -2678,17 +2761,17 @@
       <formula>"À écarter"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M27">
+  <conditionalFormatting sqref="M5:M28">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminé"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M27" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M28" type="list">
       <formula1>"À faire,En cours,Terminé"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J27" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J28" type="list">
       <formula1>"Essentielle,Utile,Optionnelle,À écarter"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2717,7 +2800,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2725,7 +2808,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2733,7 +2816,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A4)</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A4)</f>
         <v>9</v>
       </c>
     </row>
@@ -2742,7 +2825,7 @@
         <v>50</v>
       </c>
       <c r="B5" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A5)</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A5)</f>
         <v>9</v>
       </c>
     </row>
@@ -2751,8 +2834,8 @@
         <v>56</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A6)</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A6)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2760,22 +2843,22 @@
         <v>88</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$27,A7)</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A7)</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2783,16 +2866,16 @@
         <v>22</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A11&amp;"*")</f>
-        <v>14</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A11&amp;"*")</f>
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A12&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A12&amp;"*")</f>
         <v>5</v>
       </c>
     </row>
@@ -2801,16 +2884,16 @@
         <v>98</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A13&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A13&amp;"*")</f>
         <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="B14" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$27,"*"&amp;A14&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A14&amp;"*")</f>
         <v>6</v>
       </c>
     </row>
@@ -2839,63 +2922,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2903,7 +2986,7 @@
         <v>137</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2934,209 +3017,209 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -3174,12 +3257,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>246</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3187,304 +3270,304 @@
         <v>8</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>247</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>249</v>
+        <v>263</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>303</v>
+        <v>317</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>305</v>
+        <v>319</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>306</v>
+        <v>320</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>313</v>
+        <v>327</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>310</v>
+        <v>324</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>317</v>
+        <v>331</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>318</v>
+        <v>332</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>320</v>
+        <v>334</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -3529,200 +3612,200 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>322</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>324</v>
+        <v>338</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>325</v>
+        <v>339</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>326</v>
+        <v>340</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>327</v>
+        <v>341</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>328</v>
+        <v>342</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>329</v>
+        <v>343</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>330</v>
+        <v>344</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>331</v>
+        <v>345</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>332</v>
+        <v>346</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>333</v>
+        <v>347</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>334</v>
+        <v>348</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>335</v>
+        <v>349</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>336</v>
+        <v>350</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>337</v>
+        <v>351</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>338</v>
+        <v>352</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>339</v>
+        <v>353</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>340</v>
+        <v>354</v>
       </c>
       <c r="I5" s="21" t="n">
         <v>46322</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>342</v>
+        <v>356</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>343</v>
+        <v>357</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>344</v>
+        <v>358</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>46322</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>345</v>
+        <v>359</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>346</v>
+        <v>360</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>347</v>
+        <v>361</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>348</v>
+        <v>362</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>349</v>
+        <v>363</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>350</v>
+        <v>364</v>
       </c>
       <c r="I6" s="21" t="n">
         <v>46324</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>351</v>
+        <v>365</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>352</v>
+        <v>366</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>353</v>
+        <v>367</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>356</v>
+        <v>370</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>358</v>
+        <v>372</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>359</v>
+        <v>373</v>
       </c>
       <c r="I7" s="21"/>
       <c r="J7" s="16" t="s">
-        <v>360</v>
+        <v>374</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>361</v>
+        <v>375</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>362</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>363</v>
+        <v>377</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>365</v>
+        <v>379</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>366</v>
+        <v>380</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>367</v>
+        <v>381</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>368</v>
+        <v>382</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>369</v>
+        <v>383</v>
       </c>
       <c r="I8" s="21" t="n">
         <v>46321</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>370</v>
+        <v>384</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>371</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dictionnaire : onglets « Techniques de collecte » et « GSOD et GHCNh »
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -11,9 +11,11 @@
     <sheet name="Dictionnaire de données" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Synthèse" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Vérification CGU" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Vérification CGU sources" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Journal des incidents" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Techniques de collecte" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="GSOD et GHCNh" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Vérification CGU" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Vérification CGU sources" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Journal des incidents" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="441">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -664,6 +666,171 @@
   </si>
   <si>
     <t xml:space="preserve">Endpoints NOAA pour les protons et les taches solaires, accès et licence GFZ/OMNIWeb, unités exactes de chaque flux.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AuroraCast – Techniques de collecte (C1.1.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mis à jour le 29/10/2026. GHCNh : accès HTTP aux fichiers du service NOAA Open Data (classé « API » dans les manifestes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Données collectées</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accès</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fréquence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA SWPC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kp observé et prévu, Kp minute, vent solaire temps réel (Bz, vitesse, densité), échelles NOAA, alertes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">services.swpc.noaa.gov (JSON)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/auroracast/collect/noaa.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA GHCNh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observations horaires des 3 stations : nuages, température, humidité, pression, vent, visibilité, temps présent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">noaa-ghcnh-pds.s3.amazonaws.com (fichiers annuels par station)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/auroracast/collect/ghcnh.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chaque jour (lignes nouvelles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prévision à 3 jours rédigée, indices géomagnétiques du jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">services.swpc.noaa.gov/text/ (fichiers texte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crawling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMNIWeb (NASA SPDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vent solaire et champ magnétique interplanétaire horaires depuis 2010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spdf.gsfc.nasa.gov/pub/data/omni/low_res_omni/ (parcours de l'index)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/auroracast/collect/omni.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backfill à la demande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOAA GSOD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Météo quotidienne 2010 → 24/08/2025 : température, rosée, visibilité, brouillard, vent, précipitations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BigQuery bigquery-public-data.noaa_gsod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/auroracast/collect/gsod.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backfill à la demande (base figée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GFZ Potsdam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kp, ap, Ap, taches solaires et flux F10.7 depuis 1932</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kp.gfz.de (Kp_ap_Ap_SN_F107_since_1932.txt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/auroracast/collect/gfz.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synthèse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre de sources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Météo au sol : deux sources pour les mêmes stations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrôle croisé de la température moyenne du jour : écart moyen de 0,03 à 0,09 °C selon le lieu (rapport de qualité du 29/10/2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GSOD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GHCNh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accès HTTP aux fichiers (classé API)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Une mesure par jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Une mesure par heure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Période</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2010 → 24/08/2025, base figée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2010 → environ 3 jours avant la date du jour, mise à jour quotidienne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table propre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weather_daily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weather_hourly (et cloud_hourly pour les nuages)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rôle dans le projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecte SQL sur une base existante (C1.1.2) et contrôle croisé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Météo récente et horaire pour le modèle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TROMSO (010260), KIRUNA (020440), ROVANIEMI RAUTATIEASEMA (028470)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TROMSO (NOM00001026), aéroport de Kiruna (SWI0000ESNQ), gare de Rovaniemi (FIM00002847)</t>
   </si>
   <si>
     <t xml:space="preserve">Vérification juridique : SpaceWeatherLive</t>
@@ -1255,15 +1422,15 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF595959"/>
+      <b val="true"/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1332,7 +1499,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1401,20 +1568,28 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -3005,6 +3180,358 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>240</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>244</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>246</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="20" t="n">
+        <f aca="false">COUNTIF($A$5:$A$10,A14)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <f aca="false">COUNTIF($A$5:$A$10,A15)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="B16" s="20" t="n">
+        <f aca="false">COUNTIF($A$5:$A$10,A16)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="B17" s="20" t="n">
+        <f aca="false">COUNTIF($A$5:$A$10,A17)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="B18" s="20" t="n">
+        <f aca="false">COUNTIF($A$5:$A$10,A18)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="B19" s="19" t="n">
+        <f aca="false">SUM(B14:B18)</f>
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="56"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="18" t="s">
+        <v>251</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>254</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>259</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>260</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>266</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>267</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3017,214 +3544,214 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>213</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>214</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
-        <v>215</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>216</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>217</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>218</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>219</v>
+      <c r="A4" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>220</v>
+        <v>275</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>221</v>
+        <v>276</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>222</v>
+        <v>277</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>223</v>
+        <v>278</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>224</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>220</v>
+        <v>275</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>221</v>
+        <v>276</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>225</v>
+        <v>280</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>226</v>
+        <v>281</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>227</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>220</v>
+        <v>275</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>221</v>
+        <v>276</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>228</v>
+        <v>283</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>229</v>
+        <v>284</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>230</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>231</v>
+        <v>286</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>232</v>
+        <v>287</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>233</v>
+        <v>288</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>234</v>
+        <v>289</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>235</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>236</v>
+        <v>291</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>237</v>
+        <v>292</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>238</v>
+        <v>293</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>239</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>240</v>
+        <v>295</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>241</v>
+        <v>296</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>242</v>
+        <v>297</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>243</v>
+        <v>298</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>244</v>
+        <v>299</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>240</v>
+        <v>295</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>241</v>
+        <v>296</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>245</v>
+        <v>300</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>246</v>
+        <v>301</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>247</v>
+        <v>302</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>240</v>
+        <v>295</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>241</v>
+        <v>296</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>248</v>
+        <v>303</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>249</v>
+        <v>304</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>250</v>
+        <v>305</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>240</v>
+        <v>295</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>241</v>
+        <v>296</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>251</v>
+        <v>306</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>252</v>
+        <v>307</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>253</v>
+        <v>308</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>240</v>
+        <v>295</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>241</v>
+        <v>296</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>254</v>
+        <v>309</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>255</v>
+        <v>310</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>256</v>
+        <v>311</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
-        <v>257</v>
+      <c r="A16" s="21" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>258</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
+      <c r="A17" s="22" t="s">
+        <v>313</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3240,7 +3767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3257,322 +3784,322 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>259</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>260</v>
+      <c r="A2" s="17" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="17" t="s">
-        <v>215</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>216</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>218</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>261</v>
+      <c r="B4" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>262</v>
+        <v>317</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>263</v>
+        <v>318</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>264</v>
+        <v>319</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>265</v>
+        <v>320</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>266</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>262</v>
+        <v>317</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>267</v>
+        <v>322</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>268</v>
+        <v>323</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>269</v>
+        <v>324</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>270</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>262</v>
+        <v>317</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>271</v>
+        <v>326</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>272</v>
+        <v>327</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>273</v>
+        <v>328</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>274</v>
+        <v>329</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>275</v>
+        <v>330</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>276</v>
+        <v>331</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>277</v>
+        <v>332</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>278</v>
+        <v>333</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>275</v>
+        <v>330</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>280</v>
+        <v>335</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>283</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>275</v>
+        <v>330</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>285</v>
+        <v>340</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>287</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>289</v>
+        <v>344</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>291</v>
+        <v>346</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>292</v>
+        <v>347</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>293</v>
+        <v>348</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>294</v>
+        <v>349</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>295</v>
+        <v>350</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>296</v>
+        <v>351</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>297</v>
+        <v>352</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>298</v>
+        <v>353</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>299</v>
+        <v>354</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>300</v>
+        <v>355</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>301</v>
+        <v>356</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>302</v>
+        <v>357</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>303</v>
+        <v>358</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>304</v>
+        <v>359</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>305</v>
+        <v>360</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>301</v>
+        <v>356</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>306</v>
+        <v>361</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>307</v>
+        <v>362</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>308</v>
+        <v>363</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>309</v>
+        <v>364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
-        <v>310</v>
+      <c r="A16" s="21" t="s">
+        <v>365</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>311</v>
+        <v>366</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>312</v>
+        <v>367</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>313</v>
+        <v>368</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>314</v>
+        <v>369</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>315</v>
+        <v>370</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>316</v>
+        <v>371</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>317</v>
+        <v>372</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>318</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>319</v>
+        <v>374</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>321</v>
+        <v>376</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>322</v>
+        <v>377</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>323</v>
+        <v>378</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>325</v>
+        <v>380</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>326</v>
+        <v>381</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>327</v>
+        <v>382</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>328</v>
+        <v>383</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>329</v>
+        <v>384</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>330</v>
+        <v>385</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>331</v>
+        <v>386</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>332</v>
+        <v>387</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>333</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
-        <v>257</v>
+      <c r="A23" s="21" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
-        <v>334</v>
-      </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
+      <c r="A24" s="22" t="s">
+        <v>389</v>
+      </c>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3588,7 +4115,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3612,200 +4139,200 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>335</v>
+        <v>390</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>336</v>
+      <c r="A2" s="17" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
-        <v>337</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>338</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>339</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>340</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>341</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>342</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>343</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>344</v>
-      </c>
-      <c r="I4" s="17" t="s">
-        <v>345</v>
-      </c>
-      <c r="J4" s="17" t="s">
+      <c r="A4" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>394</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>395</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>397</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>398</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="J4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="17" t="s">
-        <v>346</v>
-      </c>
-      <c r="L4" s="17" t="s">
-        <v>347</v>
+      <c r="K4" s="18" t="s">
+        <v>401</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>348</v>
-      </c>
-      <c r="B5" s="21" t="n">
+        <v>403</v>
+      </c>
+      <c r="B5" s="23" t="n">
         <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>349</v>
+        <v>404</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>350</v>
+        <v>405</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>351</v>
+        <v>406</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>352</v>
+        <v>407</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>353</v>
+        <v>408</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>354</v>
-      </c>
-      <c r="I5" s="21" t="n">
+        <v>409</v>
+      </c>
+      <c r="I5" s="23" t="n">
         <v>46322</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>356</v>
+        <v>411</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>357</v>
+        <v>412</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>358</v>
-      </c>
-      <c r="B6" s="21" t="n">
+        <v>413</v>
+      </c>
+      <c r="B6" s="23" t="n">
         <v>46322</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>359</v>
+        <v>414</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>360</v>
+        <v>415</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>361</v>
+        <v>416</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>362</v>
+        <v>417</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>363</v>
+        <v>418</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>364</v>
-      </c>
-      <c r="I6" s="21" t="n">
+        <v>419</v>
+      </c>
+      <c r="I6" s="23" t="n">
         <v>46324</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>365</v>
+        <v>420</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>366</v>
+        <v>421</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>367</v>
-      </c>
-      <c r="B7" s="21" t="n">
+        <v>422</v>
+      </c>
+      <c r="B7" s="23" t="n">
         <v>46321</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>368</v>
+        <v>423</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>369</v>
+        <v>424</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>370</v>
+        <v>425</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>371</v>
+        <v>426</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>372</v>
+        <v>427</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>373</v>
-      </c>
-      <c r="I7" s="21"/>
+        <v>428</v>
+      </c>
+      <c r="I7" s="23"/>
       <c r="J7" s="16" t="s">
-        <v>374</v>
+        <v>429</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>375</v>
+        <v>430</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>376</v>
+        <v>431</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>377</v>
-      </c>
-      <c r="B8" s="21" t="n">
+        <v>432</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>46321</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>378</v>
+        <v>433</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>379</v>
+        <v>434</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>381</v>
+        <v>436</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>382</v>
+        <v>437</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>383</v>
-      </c>
-      <c r="I8" s="21" t="n">
+        <v>438</v>
+      </c>
+      <c r="I8" s="23" t="n">
         <v>46321</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>384</v>
+        <v>439</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>385</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prévisions MET Norway : table weather_forecast, notebook 04, documentation et dictionnaire
- transform/forecast.py : toutes les prévisions émises (issued_at, target_time, échéance),
  nébulosité par étage, brouillard, température, humidité, vent, pluie
- collecte : coordonnées tronquées en décimal (25.7294 devenait 25.7293)
- notebook 04 : dernière prévision horaire par lieu (nuages, brouillard, étages)
- dictionnaire : CGU et robots.txt MET Norway, 2 variables prévues, technique API

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="467">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -359,22 +359,22 @@
     <t xml:space="preserve">Horaire</t>
   </si>
   <si>
-    <t xml:space="preserve">1 fois par jour (prévision + observé de la veille)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOAA GHCNh (stations TROMSO, aéroport de Kiruna, gare de Rovaniemi) ; Open-Meteo écarté (robots.txt, INC-002)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API (fichiers annuels)</t>
+    <t xml:space="preserve">Observé : chaque jour (GHCNh) ; prévu : toutes les 3 h (MET Norway)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observé : NOAA GHCNh (stations TROMSO, aéroport de Kiruna, gare de Rovaniemi) ; prévu : MET Norway Locationforecast 2.0 (nébulosité totale et par étage) ; Open-Meteo écarté (robots.txt, INC-002)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API (fichiers GHCNh + API MET Norway)</t>
   </si>
   <si>
     <t xml:space="preserve">Un ciel couvert empêche de voir l'aurore</t>
   </si>
   <si>
-    <t xml:space="preserve">NOAA GHCNh : CC0 (citer NOAA NCEI, DOI 10.25921/jp3d-3v19)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Historique collecté (NOAA GHCNh 2010 → 24/10/2026) ; prévisions à faire</t>
+    <t xml:space="preserve">NOAA GHCNh : CC0 (DOI 10.25921/jp3d-3v19) ; MET Norway : CC BY 4.0 (citer MET Norway)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observé collecté et nettoyé (cloud_hourly, 2010 → J-3) ; prévu collecté toutes les 3 h (weather_forecast)</t>
   </si>
   <si>
     <t xml:space="preserve">Régions de taches solaires</t>
@@ -497,7 +497,7 @@
     <t xml:space="preserve">NOAA NCEI GSOD : données publiques, sans garantie (citer NCEI) ; NOAA GHCNh : CC0 (DOI 10.25921/jp3d-3v19) ; requêtes BigQuery gratuites jusqu'à 1 To par mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecté et nettoyé : GSOD (weather_daily) et GHCNh (weather_hourly, mis à jour chaque jour) ; contrôle croisé de la température : écart moyen 0,03 à 0,09 °C ; prévisions à faire</t>
+    <t xml:space="preserve">Collecté et nettoyé : GSOD (weather_daily) et GHCNh (weather_hourly, mis à jour chaque jour) ; contrôle croisé de la température : écart moyen 0,03 à 0,09 °C ; prévisions collectées (MET Norway, weather_forecast)</t>
   </si>
   <si>
     <t xml:space="preserve">Point de rosée et humidité relative</t>
@@ -572,7 +572,7 @@
     <t xml:space="preserve">NOAA NCEI : données publiques, sans garantie (citer « Global Surface Summary of the Day - GSOD », NCEI) ; requêtes BigQuery gratuites jusqu'à 1 To par mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Historique collecté et nettoyé (2010 → 24/08/2025, table weather_daily) ; prévisions à faire</t>
+    <t xml:space="preserve">Historique collecté et nettoyé (2010 → 24/08/2025, table weather_daily) ; prévisions collectées (MET Norway, weather_forecast)</t>
   </si>
   <si>
     <t xml:space="preserve">Pression au niveau de la mer</t>
@@ -599,7 +599,46 @@
     <t xml:space="preserve">NOAA GHCNh : CC0 (DOI 10.25921/jp3d-3v19)</t>
   </si>
   <si>
-    <t xml:space="preserve">Collecté et nettoyé (weather_hourly, 2010 → hier) ; prévisions à faire</t>
+    <t xml:space="preserve">Collecté et nettoyé (weather_hourly, 2010 → hier) ; prévisions collectées (MET Norway, weather_forecast)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prévision de brouillard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part de la zone autour du lieu couverte de brouillard (visibilité sous 1 km) ; seul indicateur de visibilité prévu par l'API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horaire, environ 60 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toutes les 3 h (dans le respect de l'en-tête Expires)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET Norway Locationforecast 2.0 (complete), fog_area_fraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Court terme (0 à 60 h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le brouillard masque le ciel comme les nuages ; complète la nébulosité prévue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET Norway : CC BY 4.0 (citer MET Norway, lien vers la licence)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecté toutes les 3 h (weather_forecast)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prévision de nébulosité par étage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuages bas (&lt; 2 000 m), moyens (2 000 à 5 000 m) et hauts (&gt; 5 000 m), en plus de la nébulosité totale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET Norway Locationforecast 2.0 (complete), cloud_area_fraction_low/medium/high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un voile de nuages hauts laisse parfois voir une aurore intense, pas des nuages bas</t>
   </si>
   <si>
     <t xml:space="preserve">Synthèse des variables</t>
@@ -716,6 +755,21 @@
     <t xml:space="preserve">Chaque jour (lignes nouvelles)</t>
   </si>
   <si>
+    <t xml:space="preserve">MET Norway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prévisions locales : nébulosité totale et par étage, brouillard, température, humidité, vent, pluie (horaire sur environ 50 h, puis 6 h jusqu'à 10 jours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">api.met.no/weatherapi/locationforecast/2.0/complete (JSON)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/auroracast/collect/metno.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toutes les 3 h (Expires respecté)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Prévision à 3 jours rédigée, indices géomagnétiques du jour</t>
   </si>
   <si>
@@ -971,7 +1025,7 @@
     <t xml:space="preserve">Le scraping de valeurs numériques brutes (Kp, flux, taches solaires) n'est pas interdit par les CGU, à condition de citer les sources d'origine. À éviter : graphiques, images, mise en page. Le robots.txt l'autorise pour un robot générique avec un délai de 5 secondes entre requêtes, mais refuse l'entraînement d'IA (ai-train=no) : pour un modèle de ML, prendre NOAA et GFZ à la source ou demander l'accord du site. Bonnes pratiques : une collecte par heure, 5 secondes entre pages, User-Agent identifiable. Pages lues via un outil de résumé : relire les textes sur le site avant de les citer. Vérification faite le 26/10/2026, ce n'est pas un avis juridique.</t>
   </si>
   <si>
-    <t xml:space="preserve">Vérification juridique : GFZ, NOAA SWPC, OMNIWeb (NASA), Open-Meteo, NOAA GHCNh, NOAA GSOD (BigQuery)</t>
+    <t xml:space="preserve">Vérification juridique : GFZ, NOAA SWPC, OMNIWeb (NASA), Open-Meteo, NOAA GHCNh, NOAA GSOD (BigQuery), MET Norway</t>
   </si>
   <si>
     <t xml:space="preserve">Vérification faite le 26/10/2026 (C1.1.2, cadre réglementaire). Ce n'est pas un avis juridique. Pages lues via un outil de résumé : relire les textes sur les sites avant de les citer.</t>
@@ -1193,10 +1247,34 @@
     <t xml:space="preserve">Mode sandbox, sans carte bancaire. Chaque requête est d'abord estimée à blanc puis plafonnée à 15 Go (la plus grosse lit 8,7 Go). Compte de service limité au rôle « Utilisateur de job BigQuery ».</t>
   </si>
   <si>
+    <t xml:space="preserve">MET Norway (prévisions météo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conditions d'utilisation de l'API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://api.met.no/doc/TermsOfService</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User-Agent identifiable avec contact obligatoire ; plus de 20 requêtes par seconde : accord spécial, sinon HTTP 429 ; ne pas redemander avant l'en-tête Expires, utiliser If-Modified-Since ; coordonnées à 4 décimales au plus (5 : HTTP 403) ; données ouvertes sous CC BY 4.0 (citer, lien vers la licence, signaler les modifications) ; interdit de contourner les limites ou d'usurper un autre client, sous peine de blocage définitif.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 requêtes toutes les 3 h, User-Agent « AuroraCast » avec contact, Expires et If-Modified-Since lus dans les manifestes, coordonnées tronquées à 4 décimales (en décimal). Citer « Données MET Norway, CC BY 4.0 » dans l'application et le dossier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://api.met.no/robots.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Googlebot et AdsBot-Google : seule la documentation est permise, /weatherapi/* interdit. « User-agent: * » : Disallow vide, donc tout est permis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collecte autorisée pour AuroraCast ; vérifié automatiquement à chaque passage (manifeste : robots = « lu », allowed = true).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Toutes les sources</t>
   </si>
   <si>
-    <t xml:space="preserve">GFZ, NOAA SWPC, OMNIWeb, NOAA GHCNh et NOAA GSOD (via BigQuery) autorisent la collecte et la réutilisation pour un projet de certification, à condition de les citer. Open-Meteo est écarté : le robots.txt de son API d'archive interdit l'accès (incident INC-002). Restriction d'usage commercial à retenir : le nombre de taches solaires du fichier GFZ (CC BY-NC 4.0). Obligation d'affichage : une prévision présentée comme celle d'AuroraCast, pas de la NOAA. Coût BigQuery : nul tant que les requêtes restent sous 1 To par mois. Le respect du robots.txt est contrôlé automatiquement à chaque collecte.</t>
+    <t xml:space="preserve">GFZ, NOAA SWPC, OMNIWeb, NOAA GHCNh, NOAA GSOD (via BigQuery) et MET Norway autorisent la collecte et la réutilisation pour un projet de certification, à condition de les citer. Open-Meteo est écarté : le robots.txt de son API d'archive interdit l'accès (incident INC-002). Restriction d'usage commercial à retenir : le nombre de taches solaires du fichier GFZ (CC BY-NC 4.0). Obligations d'affichage : une prévision présentée comme celle d'AuroraCast, pas de la NOAA ; mention « Données MET Norway, CC BY 4.0 » à côté des prévisions météo. Coût BigQuery : nul tant que les requêtes restent sous 1 To par mois. Le respect du robots.txt est contrôlé automatiquement à chaque collecte.</t>
   </si>
   <si>
     <t xml:space="preserve">Journal des incidents de collecte</t>
@@ -1499,7 +1577,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1574,10 +1652,6 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1871,7 +1945,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -2924,8 +2998,90 @@
         <v>190</v>
       </c>
     </row>
+    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="J30" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="M30" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J5:J28">
+  <conditionalFormatting sqref="J5:J30">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Essentielle"</formula>
     </cfRule>
@@ -2936,17 +3092,17 @@
       <formula>"À écarter"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M28">
+  <conditionalFormatting sqref="M5:M30">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminé"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M28" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M30" type="list">
       <formula1>"À faire,En cours,Terminé"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J28" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J30" type="list">
       <formula1>"Essentielle,Utile,Optionnelle,À écarter"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2975,7 +3131,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2983,7 +3139,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2991,8 +3147,8 @@
         <v>24</v>
       </c>
       <c r="B4" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A4)</f>
-        <v>9</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$30,A4)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3000,8 +3156,8 @@
         <v>50</v>
       </c>
       <c r="B5" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A5)</f>
-        <v>9</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$30,A5)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3009,7 +3165,7 @@
         <v>56</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A6)</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$30,A6)</f>
         <v>5</v>
       </c>
     </row>
@@ -3018,22 +3174,22 @@
         <v>88</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$28,A7)</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$J$5:$J$30,A7)</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3041,16 +3197,16 @@
         <v>22</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A11&amp;"*")</f>
-        <v>20</v>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$30,"*"&amp;A11&amp;"*")</f>
+        <v>22</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A12&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$30,"*"&amp;A12&amp;"*")</f>
         <v>5</v>
       </c>
     </row>
@@ -3059,16 +3215,16 @@
         <v>98</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A13&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$30,"*"&amp;A13&amp;"*")</f>
         <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="B14" s="10" t="n">
-        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$28,"*"&amp;A14&amp;"*")</f>
+        <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$30,"*"&amp;A14&amp;"*")</f>
         <v>6</v>
       </c>
     </row>
@@ -3097,63 +3253,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3161,7 +3317,7 @@
         <v>137</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -3180,232 +3336,253 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
         <v>22</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="F6" s="16" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>244</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>253</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>255</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>258</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
+        <v>260</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>261</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>229</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>230</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>223</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
-        <v>231</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>232</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>234</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>235</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>237</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>239</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>240</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>243</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>244</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>245</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+      <c r="B14" s="13" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="20" t="n">
-        <f aca="false">COUNTIF($A$5:$A$10,A14)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="B15" s="20" t="n">
-        <f aca="false">COUNTIF($A$5:$A$10,A15)</f>
+      <c r="B15" s="19" t="n">
+        <f aca="false">COUNTIF($A$5:$A$11,A15)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <f aca="false">COUNTIF($A$5:$A$11,A16)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>231</v>
-      </c>
-      <c r="B16" s="20" t="n">
-        <f aca="false">COUNTIF($A$5:$A$10,A16)</f>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <f aca="false">COUNTIF($A$5:$A$11,A17)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
-        <v>196</v>
-      </c>
-      <c r="B17" s="20" t="n">
-        <f aca="false">COUNTIF($A$5:$A$10,A17)</f>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <f aca="false">COUNTIF($A$5:$A$11,A18)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
-        <v>242</v>
-      </c>
-      <c r="B18" s="20" t="n">
-        <f aca="false">COUNTIF($A$5:$A$10,A18)</f>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="B19" s="19" t="n">
+        <f aca="false">COUNTIF($A$5:$A$11,A19)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="B19" s="19" t="n">
-        <f aca="false">SUM(B14:B18)</f>
-        <v>6</v>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="B20" s="13" t="n">
+        <f aca="false">SUM(B15:B19)</f>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -3427,93 +3604,93 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="56"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>250</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="18" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="B5" s="16" t="s">
         <v>178</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>262</v>
+        <v>280</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>266</v>
+        <v>284</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>267</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -3544,214 +3721,214 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>279</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>282</v>
+        <v>300</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>285</v>
+        <v>303</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>286</v>
+        <v>304</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>288</v>
+        <v>306</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>289</v>
+        <v>307</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>290</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>291</v>
+        <v>309</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>292</v>
+        <v>310</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>293</v>
+        <v>311</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>298</v>
+        <v>316</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>302</v>
+        <v>320</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>304</v>
+        <v>322</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>312</v>
+      <c r="A16" s="20" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
-        <v>313</v>
-      </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
+      <c r="A17" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3772,7 +3949,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -3784,12 +3961,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3797,313 +3974,347 @@
         <v>8</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>316</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>319</v>
+        <v>337</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>322</v>
+        <v>340</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>323</v>
+        <v>341</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>324</v>
+        <v>342</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>326</v>
+        <v>344</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>353</v>
+        <v>371</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>354</v>
+        <v>372</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>355</v>
+        <v>373</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>357</v>
+        <v>375</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>358</v>
+        <v>376</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>359</v>
+        <v>377</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>360</v>
+        <v>378</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>361</v>
+        <v>379</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>362</v>
+        <v>380</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>363</v>
+        <v>381</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>364</v>
+        <v>382</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>365</v>
+      <c r="A16" s="20" t="s">
+        <v>383</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>366</v>
+        <v>384</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>367</v>
+        <v>385</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>370</v>
+        <v>388</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>371</v>
+        <v>389</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>372</v>
+        <v>390</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>373</v>
+        <v>391</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>374</v>
+        <v>392</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>375</v>
+        <v>393</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>377</v>
+        <v>395</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>378</v>
+        <v>396</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>380</v>
+        <v>398</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>381</v>
+        <v>399</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>382</v>
+        <v>400</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>383</v>
+        <v>401</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>384</v>
+        <v>402</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>386</v>
+        <v>404</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+        <v>406</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>407</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>408</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="s">
+        <v>406</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>411</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>412</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>413</v>
+      </c>
+    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22" t="s">
-        <v>389</v>
-      </c>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
+      <c r="A23" s="16" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
+        <v>415</v>
+      </c>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A26:E26"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4139,200 +4350,200 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>390</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>391</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>392</v>
+        <v>418</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>394</v>
+        <v>420</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>395</v>
+        <v>421</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>396</v>
+        <v>422</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>397</v>
+        <v>423</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>398</v>
+        <v>424</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>399</v>
+        <v>425</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>400</v>
+        <v>426</v>
       </c>
       <c r="J4" s="18" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>401</v>
+        <v>427</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>402</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>403</v>
-      </c>
-      <c r="B5" s="23" t="n">
+        <v>429</v>
+      </c>
+      <c r="B5" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>404</v>
+        <v>430</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>405</v>
+        <v>431</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>406</v>
+        <v>432</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>407</v>
+        <v>433</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>408</v>
+        <v>434</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>409</v>
-      </c>
-      <c r="I5" s="23" t="n">
+        <v>435</v>
+      </c>
+      <c r="I5" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>410</v>
+        <v>436</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>411</v>
+        <v>437</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>412</v>
+        <v>438</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>413</v>
-      </c>
-      <c r="B6" s="23" t="n">
+        <v>439</v>
+      </c>
+      <c r="B6" s="22" t="n">
         <v>46322</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>414</v>
+        <v>440</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>415</v>
+        <v>441</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>416</v>
+        <v>442</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>417</v>
+        <v>443</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>418</v>
+        <v>444</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>419</v>
-      </c>
-      <c r="I6" s="23" t="n">
+        <v>445</v>
+      </c>
+      <c r="I6" s="22" t="n">
         <v>46324</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>410</v>
+        <v>436</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>420</v>
+        <v>446</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>421</v>
+        <v>447</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>422</v>
-      </c>
-      <c r="B7" s="23" t="n">
+        <v>448</v>
+      </c>
+      <c r="B7" s="22" t="n">
         <v>46321</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>423</v>
+        <v>449</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>424</v>
+        <v>450</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>425</v>
+        <v>451</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>426</v>
+        <v>452</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>427</v>
+        <v>453</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>428</v>
-      </c>
-      <c r="I7" s="23"/>
+        <v>454</v>
+      </c>
+      <c r="I7" s="22"/>
       <c r="J7" s="16" t="s">
-        <v>429</v>
+        <v>455</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>430</v>
+        <v>456</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>431</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>432</v>
-      </c>
-      <c r="B8" s="23" t="n">
+        <v>458</v>
+      </c>
+      <c r="B8" s="22" t="n">
         <v>46321</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>433</v>
+        <v>459</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>434</v>
+        <v>460</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>435</v>
+        <v>461</v>
       </c>
       <c r="F8" s="16" t="s">
+        <v>462</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>463</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>464</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>46321</v>
+      </c>
+      <c r="J8" s="16" t="s">
         <v>436</v>
       </c>
-      <c r="G8" s="16" t="s">
-        <v>437</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>438</v>
-      </c>
-      <c r="I8" s="23" t="n">
-        <v>46321</v>
-      </c>
-      <c r="J8" s="16" t="s">
-        <v>410</v>
-      </c>
       <c r="K8" s="16" t="s">
-        <v>439</v>
+        <v>465</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>440</v>
+        <v>466</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Table astronomique astronomy_hourly (PyEphem) et notebook 05
- hauteur du Soleil et phase de la nuit, hauteur et éclairement de la Lune, nuit polaire et
  soleil de minuit, par lieu et par heure, 2010 -> J+10 ; vérifié contre sunrise-sunset.org
- notebook 05 : heures de ciel noir par jour, vérification de l'anomalie de Tromsø (le noir
  n'explique pas le ciel dégagé de janvier ; « 0 octa » 2 fois plus fréquent de nuit)
- dictionnaire et README à jour ; dépendance ephem

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="471">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -308,19 +308,19 @@
     <t xml:space="preserve">Calculée</t>
   </si>
   <si>
-    <t xml:space="preserve">Pourcentage d'illumination de la Lune ; une pleine Lune gêne la visibilité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% (0 à 100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calcul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculée à la demande</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bibliothèque astral / ephem</t>
+    <t xml:space="preserve">Hauteur de la Lune au-dessus de l'horizon et part du disque éclairé ; une Lune haute et pleine efface les aurores faibles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">degrés / % (0 à 100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horaire (calcul)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recalculée à chaque transformation (2010 → J+10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PyEphem 4.2 (licence MIT, éphémérides intégrées, aucun téléchargement)</t>
   </si>
   <si>
     <t xml:space="preserve">Calcul local</t>
@@ -329,21 +329,30 @@
     <t xml:space="preserve">N'influence pas l'aurore mais la visibilité</t>
   </si>
   <si>
-    <t xml:space="preserve">Sans objet (calcul)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nuit noire (début/fin)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Période de nuit astronomique pour un lieu donné</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heure locale</t>
+    <t xml:space="preserve">Sans objet (calcul) ; PyEphem sous licence MIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculé (astronomy_hourly : moon_alt_deg, moon_illum_pct, moon_up)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuit noire et hauteur du Soleil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hauteur géométrique du Soleil et phase de la nuit : jour, crépuscule civil (jusqu'à -6°), nautique (-12°), astronomique (-18°), nuit ; nuit polaire et soleil de minuit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">degrés / catégorie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PyEphem 4.2 (licence MIT) ; vérifié contre sunrise-sunset.org (Tromsø, 29/10/2026 : écart &lt; 5 s)</t>
   </si>
   <si>
     <t xml:space="preserve">Condition de visibilité de l'aurore</t>
   </si>
   <si>
+    <t xml:space="preserve">Calculé (astronomy_hourly : sun_alt_deg, night_phase, polar_night, midnight_sun)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nébulosité</t>
   </si>
   <si>
@@ -822,6 +831,9 @@
   </si>
   <si>
     <t xml:space="preserve">src/auroracast/collect/gfz.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hors collecte : la table astronomique (Soleil, Lune, nuit polaire) est calculée localement avec PyEphem, sans source externe (src/auroracast/transform/astronomy.py).</t>
   </si>
   <si>
     <t xml:space="preserve">Synthèse</t>
@@ -1577,7 +1589,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1652,6 +1664,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -2462,21 +2478,21 @@
         <v>100</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>92</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>95</v>
@@ -2485,7 +2501,7 @@
         <v>96</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>98</v>
@@ -2497,39 +2513,39 @@
         <v>24</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="L16" s="6" t="s">
         <v>100</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I17" s="7" t="s">
         <v>23</v>
@@ -2538,39 +2554,39 @@
         <v>24</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>33</v>
@@ -2579,10 +2595,10 @@
         <v>50</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>90</v>
@@ -2590,16 +2606,16 @@
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>40</v>
@@ -2608,10 +2624,10 @@
         <v>72</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>49</v>
@@ -2620,7 +2636,7 @@
         <v>50</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="L19" s="6" t="s">
         <v>35</v>
@@ -2631,28 +2647,28 @@
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I20" s="7" t="s">
         <v>49</v>
@@ -2661,10 +2677,10 @@
         <v>56</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>90</v>
@@ -2672,69 +2688,69 @@
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>78</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>50</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="L21" s="6" t="s">
         <v>35</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>23</v>
@@ -2743,39 +2759,39 @@
         <v>50</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>49</v>
@@ -2784,39 +2800,39 @@
         <v>50</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I24" s="7" t="s">
         <v>49</v>
@@ -2825,39 +2841,39 @@
         <v>24</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M24" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>49</v>
@@ -2866,39 +2882,39 @@
         <v>24</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>49</v>
@@ -2907,39 +2923,39 @@
         <v>56</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>49</v>
@@ -2948,39 +2964,39 @@
         <v>56</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>49</v>
@@ -2989,95 +3005,95 @@
         <v>56</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="M28" s="7" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>24</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>50</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="M30" s="7" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -3131,7 +3147,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3139,7 +3155,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3180,7 +3196,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM(B4:B7)</f>
@@ -3189,7 +3205,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3203,7 +3219,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$30,"*"&amp;A12&amp;"*")</f>
@@ -3221,7 +3237,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">COUNTIF('Dictionnaire de données'!$H$5:$H$30,"*"&amp;A14&amp;"*")</f>
@@ -3253,71 +3269,71 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -3349,32 +3365,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3382,16 +3398,16 @@
         <v>22</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>72</v>
@@ -3402,19 +3418,19 @@
         <v>22</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3422,36 +3438,36 @@
         <v>22</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>72</v>
@@ -3459,126 +3475,130 @@
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+        <v>257</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
+        <v>268</v>
+      </c>
+    </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="20" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A15)</f>
         <v>3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
-        <v>208</v>
-      </c>
-      <c r="B16" s="19" t="n">
+      <c r="A16" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="B16" s="20" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A16)</f>
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>249</v>
-      </c>
-      <c r="B17" s="19" t="n">
+      <c r="A17" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="B17" s="20" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A17)</f>
         <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="B18" s="19" t="n">
+      <c r="A18" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="B18" s="20" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A18)</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>260</v>
-      </c>
-      <c r="B19" s="19" t="n">
+      <c r="A19" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="B19" s="20" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A19)</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">SUM(B15:B19)</f>
@@ -3611,86 +3631,86 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="18" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -3721,214 +3741,214 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>330</v>
+      <c r="A16" s="21" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
-        <v>331</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
+      <c r="A17" s="22" t="s">
+        <v>335</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3961,12 +3981,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3974,343 +3994,343 @@
         <v>8</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
-        <v>383</v>
+      <c r="A16" s="21" t="s">
+        <v>387</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>330</v>
+      <c r="A25" s="21" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="s">
-        <v>415</v>
-      </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
+      <c r="A26" s="22" t="s">
+        <v>419</v>
+      </c>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4350,200 +4370,200 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="J4" s="18" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>429</v>
-      </c>
-      <c r="B5" s="22" t="n">
+        <v>433</v>
+      </c>
+      <c r="B5" s="23" t="n">
         <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>435</v>
-      </c>
-      <c r="I5" s="22" t="n">
+        <v>439</v>
+      </c>
+      <c r="I5" s="23" t="n">
         <v>46322</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>439</v>
-      </c>
-      <c r="B6" s="22" t="n">
+        <v>443</v>
+      </c>
+      <c r="B6" s="23" t="n">
         <v>46322</v>
       </c>
       <c r="C6" s="16" t="s">
+        <v>444</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>445</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>448</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>449</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>46324</v>
+      </c>
+      <c r="J6" s="16" t="s">
         <v>440</v>
       </c>
-      <c r="D6" s="16" t="s">
-        <v>441</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>442</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>443</v>
-      </c>
-      <c r="G6" s="16" t="s">
-        <v>444</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>445</v>
-      </c>
-      <c r="I6" s="22" t="n">
-        <v>46324</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>436</v>
-      </c>
       <c r="K6" s="16" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>448</v>
-      </c>
-      <c r="B7" s="22" t="n">
+        <v>452</v>
+      </c>
+      <c r="B7" s="23" t="n">
         <v>46321</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>454</v>
-      </c>
-      <c r="I7" s="22"/>
+        <v>458</v>
+      </c>
+      <c r="I7" s="23"/>
       <c r="J7" s="16" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>458</v>
-      </c>
-      <c r="B8" s="22" t="n">
+        <v>462</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>46321</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>464</v>
-      </c>
-      <c r="I8" s="22" t="n">
+        <v>468</v>
+      </c>
+      <c r="I8" s="23" t="n">
         <v>46321</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dictionnaire : onglet Entrepôt (tables, clés, contraintes, colonnes, origine) ; README : nombre de lignes exact
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4Z8zdgvPrzbs3BgLqcvsx
</commit_message>
<xml_diff>
--- a/docs/dictionnaire_donnees.xlsx
+++ b/docs/dictionnaire_donnees.xlsx
@@ -13,9 +13,10 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Techniques de collecte" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="GSOD et GHCNh" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Vérification CGU" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Vérification CGU sources" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Journal des incidents" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Entrepôt" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Vérification CGU" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Vérification CGU sources" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Journal des incidents" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="555">
   <si>
     <t xml:space="preserve">AuroraCast – Dictionnaire de données (activité aurorale et solaire)</t>
   </si>
@@ -716,6 +717,12 @@
     <t xml:space="preserve">Endpoints NOAA pour les protons et les taches solaires, accès et licence GFZ/OMNIWeb, unités exactes de chaque flux.</t>
   </si>
   <si>
+    <t xml:space="preserve">Entrepôt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toutes les tables propres sont chargées chaque jour dans PostgreSQL (onglet « Entrepôt ») : Neon dans le cloud, Docker en local.</t>
+  </si>
+  <si>
     <t xml:space="preserve">AuroraCast – Techniques de collecte (C1.1.2)</t>
   </si>
   <si>
@@ -897,6 +904,260 @@
   </si>
   <si>
     <t xml:space="preserve">TROMSO (NOM00001026), aéroport de Kiruna (SWI0000ESNQ), gare de Rovaniemi (FIM00002847)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrepôt PostgreSQL : modèle en étoile (sql/schema.sql)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Généré depuis la base le 29/10/2026 (information_schema). Hébergement : Neon (AWS US East 2), et Docker en local. Rechargement complet chaque jour, en une transaction. Lignes au chargement du 29/10/2026 (environ 213 Mo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clé primaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clés étrangères</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contraintes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colonnes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table propre d'origine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lignes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dim_location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">un lieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIQUE (code)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id, code, name, lat, lon, station_id, station_name, station_distance_km</t>
+  </si>
+  <si>
+    <t xml:space="preserve">locations (+ data/stations.json)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dim_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">une heure UTC, 1932 → J+10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">time_utc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">time_utc, date_utc, year, month, day, hour, day_of_year, iso_week, aurora_season</t>
+  </si>
+  <si>
+    <t xml:space="preserve">calculée au chargement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dim_source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">une source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source_id, code, name, technique, licence, url</t>
+  </si>
+  <si>
+    <t xml:space="preserve">liste fixe dans warehouse/load.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_kp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fait global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">time_utc → dim_time
+source_id → dim_source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK (kp &gt;= (0)) AND (kp &lt;= (9))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">time_utc, kp, ap, status, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kp_3h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_kp_forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">émission × tranche de 3 h visée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">issued_at, target_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_time → dim_time
+source_id → dim_source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">issued_at, target_time, kp, noaa_scale, lead_hours, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kp_forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_solar_daily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jour (00:00 UTC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">time_utc, ap_daily, sunspot_number, f107_obs, f107_adj, sunspot_status, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">solar_daily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_solar_wind</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">time_utc, bt, by_gsm, bz_gsm, bz_min, speed, speed_max, density, interpolated, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">solar_wind_hourly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_weather_observed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fait par lieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lieu × 1 h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id, time_utc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id → dim_location
+time_utc → dim_time
+source_id → dim_source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK (oktas &gt;= (0)) AND (oktas &lt;= (8))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id, time_utc, oktas, cloud_cover_pct, obscured, temp_c, dewpoint_c, rel_humidity_pct, pressure_hpa, wind_speed_ms, wind_dir_deg, visibility_km, visibility_capped, fog, mist, present_weather, n_obs, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cloud_hourly + weather_hourly (fusionnées)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_weather_daily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lieu × jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source_id → dim_source
+location_id → dim_location
+time_utc → dim_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id, time_utc, station_id, temp_c, temp_max_c, temp_min_c, dewpoint_c, rel_humidity_pct, visibility_km, wind_mean_ms, wind_max_ms, precip_mm, precip_flag, precip_suspect, fog, rain, snow, hail, thunder, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_weather_forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lieu × émission × heure visée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id, issued_at, target_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_time → dim_time
+location_id → dim_location
+source_id → dim_source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id, issued_at, target_time, lead_hours, step_hours, cloud_cover_pct, cloud_low_pct, cloud_medium_pct, cloud_high_pct, fog_pct, temp_c, dewpoint_c, rel_humidity_pct, pressure_hpa, wind_speed_ms, wind_dir_deg, wind_gust_ms, precip_mm, precip_probability_pct, symbol_code, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weather_forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_astronomy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location_id, time_utc, sun_alt_deg, night_phase, moon_alt_deg, moon_illum_pct, moon_up, polar_night, midnight_sun, source_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">astronomy_hourly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">load_run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">un chargement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">run_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">run_id, started_at, finished_at, rows_loaded, database_mb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">écrite par warehouse/load.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v_aurora_conditions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">location, time_utc, kp, kp_ge_4, oktas, fog, sun_alt_deg, night_phase, moon_alt_deg, moon_illum_pct, dark_sky, clear_sky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_astronomy + fact_weather_observed + fact_kp + dim_location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total des lignes (tables chargées)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombres de lignes du chargement du 29/10/2026 ; chaque chargement les enregistre dans la table load_run.</t>
   </si>
   <si>
     <t xml:space="preserve">Vérification juridique : SpaceWeatherLive</t>
@@ -1446,10 +1707,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="#,##0"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1589,7 +1851,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1666,12 +1928,24 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1682,7 +1956,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3260,7 +3534,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -3334,6 +3608,14 @@
       </c>
       <c r="B10" s="16" t="s">
         <v>228</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -3365,32 +3647,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3398,16 +3680,16 @@
         <v>22</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>72</v>
@@ -3418,19 +3700,19 @@
         <v>22</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3438,19 +3720,19 @@
         <v>22</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3458,16 +3740,16 @@
         <v>211</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>72</v>
@@ -3475,22 +3757,22 @@
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3498,100 +3780,100 @@
         <v>212</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>268</v>
+      <c r="A12" s="17" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="20" t="n">
+      <c r="B15" s="19" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A15)</f>
         <v>3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="B16" s="20" t="n">
+      <c r="B16" s="19" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A16)</f>
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="s">
-        <v>252</v>
-      </c>
-      <c r="B17" s="20" t="n">
+      <c r="A17" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="B17" s="19" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A17)</f>
         <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="19" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A18)</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
-        <v>263</v>
-      </c>
-      <c r="B19" s="20" t="n">
+      <c r="A19" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="B19" s="19" t="n">
         <f aca="false">COUNTIF($A$5:$A$11,A19)</f>
         <v>1</v>
       </c>
@@ -3631,31 +3913,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="18" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B5" s="16" t="s">
         <v>181</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3663,54 +3945,54 @@
         <v>215</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -3729,6 +4011,462 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>309</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>310</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>831490</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>320</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>321</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>324</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>325</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>326</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>277083</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>321</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>328</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>330</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>321</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>334</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>336</v>
+      </c>
+      <c r="I10" s="20" t="n">
+        <v>34633</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>321</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>338</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>339</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="I11" s="20" t="n">
+        <v>147490</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>343</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>345</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>346</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>347</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>348</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <v>442262</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>350</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>351</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="I13" s="20" t="n">
+        <v>17145</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>355</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>356</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>357</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="I14" s="20" t="n">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>343</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>345</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <v>443190</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="I16" s="20"/>
+    </row>
+    <row r="17" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>343</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="I17" s="20"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>372</v>
+      </c>
+      <c r="I19" s="22" t="n">
+        <f aca="false">SUM(I5:I17)</f>
+        <v>2193606</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="23" t="s">
+        <v>373</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3741,214 +4479,214 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>290</v>
+        <v>374</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>291</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>292</v>
+        <v>376</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>293</v>
+        <v>377</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>294</v>
+        <v>378</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>295</v>
+        <v>379</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>296</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>297</v>
+        <v>381</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>298</v>
+        <v>382</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>299</v>
+        <v>383</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>300</v>
+        <v>384</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>301</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>297</v>
+        <v>381</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>298</v>
+        <v>382</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>302</v>
+        <v>386</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>303</v>
+        <v>387</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>304</v>
+        <v>388</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>297</v>
+        <v>381</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>298</v>
+        <v>382</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>305</v>
+        <v>389</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>306</v>
+        <v>390</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>307</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>308</v>
+        <v>392</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>309</v>
+        <v>393</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>310</v>
+        <v>394</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>311</v>
+        <v>395</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>312</v>
+        <v>396</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>313</v>
+        <v>397</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>314</v>
+        <v>398</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>315</v>
+        <v>399</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>316</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>317</v>
+        <v>401</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>318</v>
+        <v>402</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>319</v>
+        <v>403</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>320</v>
+        <v>404</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>321</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>317</v>
+        <v>401</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>318</v>
+        <v>402</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>322</v>
+        <v>406</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>323</v>
+        <v>407</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>324</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>317</v>
+        <v>401</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>318</v>
+        <v>402</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>325</v>
+        <v>409</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>326</v>
+        <v>410</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>327</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>317</v>
+        <v>401</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>318</v>
+        <v>402</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>328</v>
+        <v>412</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>329</v>
+        <v>413</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>330</v>
+        <v>414</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>317</v>
+        <v>401</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>318</v>
+        <v>402</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>331</v>
+        <v>415</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>332</v>
+        <v>416</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>333</v>
+        <v>417</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>334</v>
+      <c r="A16" s="24" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
-        <v>335</v>
-      </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
+      <c r="A17" s="25" t="s">
+        <v>419</v>
+      </c>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3964,7 +4702,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3981,12 +4719,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>336</v>
+        <v>420</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>337</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3994,343 +4732,343 @@
         <v>8</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>292</v>
+        <v>376</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>293</v>
+        <v>377</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>295</v>
+        <v>379</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>338</v>
+        <v>422</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>339</v>
+        <v>423</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>340</v>
+        <v>424</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>341</v>
+        <v>425</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>342</v>
+        <v>426</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>343</v>
+        <v>427</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>339</v>
+        <v>423</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>344</v>
+        <v>428</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>345</v>
+        <v>429</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>346</v>
+        <v>430</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>347</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>339</v>
+        <v>423</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>348</v>
+        <v>432</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>349</v>
+        <v>433</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>350</v>
+        <v>434</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>351</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>352</v>
+        <v>436</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>353</v>
+        <v>437</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>354</v>
+        <v>438</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>355</v>
+        <v>439</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>356</v>
+        <v>440</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>352</v>
+        <v>436</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>357</v>
+        <v>441</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>358</v>
+        <v>442</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>359</v>
+        <v>443</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>360</v>
+        <v>444</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>352</v>
+        <v>436</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>361</v>
+        <v>445</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>362</v>
+        <v>446</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>363</v>
+        <v>447</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>364</v>
+        <v>448</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>365</v>
+        <v>449</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>366</v>
+        <v>450</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>367</v>
+        <v>451</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>368</v>
+        <v>452</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>369</v>
+        <v>453</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>365</v>
+        <v>449</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>370</v>
+        <v>454</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>371</v>
+        <v>455</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>372</v>
+        <v>456</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>373</v>
+        <v>457</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>365</v>
+        <v>449</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>374</v>
+        <v>458</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>375</v>
+        <v>459</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>376</v>
+        <v>460</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>377</v>
+        <v>461</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>378</v>
+        <v>462</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>379</v>
+        <v>463</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>380</v>
+        <v>464</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>381</v>
+        <v>465</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>382</v>
+        <v>466</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>378</v>
+        <v>462</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>383</v>
+        <v>467</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>384</v>
+        <v>468</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>385</v>
+        <v>469</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>386</v>
+        <v>470</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>387</v>
+      <c r="A16" s="24" t="s">
+        <v>471</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>388</v>
+        <v>472</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>389</v>
+        <v>473</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>390</v>
+        <v>474</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>391</v>
+        <v>475</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>387</v>
+        <v>471</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>392</v>
+        <v>476</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>393</v>
+        <v>477</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>394</v>
+        <v>478</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>395</v>
+        <v>479</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>396</v>
+        <v>480</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>397</v>
+        <v>481</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>398</v>
+        <v>482</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>399</v>
+        <v>483</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>400</v>
+        <v>484</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>401</v>
+        <v>485</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>402</v>
+        <v>486</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>403</v>
+        <v>487</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>404</v>
+        <v>488</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>405</v>
+        <v>489</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>401</v>
+        <v>485</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>406</v>
+        <v>490</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>407</v>
+        <v>491</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>408</v>
+        <v>492</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>409</v>
+        <v>493</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>410</v>
+        <v>494</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>411</v>
+        <v>495</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>412</v>
+        <v>496</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>413</v>
+        <v>497</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>414</v>
+        <v>498</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>410</v>
+        <v>494</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>317</v>
+        <v>401</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>415</v>
+        <v>499</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>416</v>
+        <v>500</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>417</v>
+        <v>501</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="s">
-        <v>418</v>
+        <v>502</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
-        <v>334</v>
+      <c r="A25" s="24" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22" t="s">
-        <v>419</v>
-      </c>
-      <c r="B26" s="22"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
+      <c r="A26" s="25" t="s">
+        <v>503</v>
+      </c>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4346,7 +5084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4370,200 +5108,200 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>420</v>
+        <v>504</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>421</v>
+        <v>505</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>422</v>
+        <v>506</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>423</v>
+        <v>507</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>424</v>
+        <v>508</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>425</v>
+        <v>509</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>426</v>
+        <v>510</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>427</v>
+        <v>511</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>428</v>
+        <v>512</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>429</v>
+        <v>513</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>430</v>
+        <v>514</v>
       </c>
       <c r="J4" s="18" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>431</v>
+        <v>515</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>432</v>
+        <v>516</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>433</v>
-      </c>
-      <c r="B5" s="23" t="n">
+        <v>517</v>
+      </c>
+      <c r="B5" s="26" t="n">
         <v>46322</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>434</v>
+        <v>518</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>435</v>
+        <v>519</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>436</v>
+        <v>520</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>437</v>
+        <v>521</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>438</v>
+        <v>522</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>439</v>
-      </c>
-      <c r="I5" s="23" t="n">
+        <v>523</v>
+      </c>
+      <c r="I5" s="26" t="n">
         <v>46322</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>440</v>
+        <v>524</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>441</v>
+        <v>525</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>442</v>
+        <v>526</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>443</v>
-      </c>
-      <c r="B6" s="23" t="n">
+        <v>527</v>
+      </c>
+      <c r="B6" s="26" t="n">
         <v>46322</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>444</v>
+        <v>528</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>445</v>
+        <v>529</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>446</v>
+        <v>530</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>447</v>
+        <v>531</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>448</v>
+        <v>532</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>449</v>
-      </c>
-      <c r="I6" s="23" t="n">
+        <v>533</v>
+      </c>
+      <c r="I6" s="26" t="n">
         <v>46324</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>440</v>
+        <v>524</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>450</v>
+        <v>534</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>451</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>452</v>
-      </c>
-      <c r="B7" s="23" t="n">
+        <v>536</v>
+      </c>
+      <c r="B7" s="26" t="n">
         <v>46321</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>453</v>
+        <v>537</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>454</v>
+        <v>538</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>455</v>
+        <v>539</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>456</v>
+        <v>540</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>457</v>
+        <v>541</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>458</v>
-      </c>
-      <c r="I7" s="23"/>
+        <v>542</v>
+      </c>
+      <c r="I7" s="26"/>
       <c r="J7" s="16" t="s">
-        <v>459</v>
+        <v>543</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>460</v>
+        <v>544</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>461</v>
+        <v>545</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>462</v>
-      </c>
-      <c r="B8" s="23" t="n">
+        <v>546</v>
+      </c>
+      <c r="B8" s="26" t="n">
         <v>46321</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>463</v>
+        <v>547</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>464</v>
+        <v>548</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>465</v>
+        <v>549</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>466</v>
+        <v>550</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>467</v>
+        <v>551</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>468</v>
-      </c>
-      <c r="I8" s="23" t="n">
+        <v>552</v>
+      </c>
+      <c r="I8" s="26" t="n">
         <v>46321</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>440</v>
+        <v>524</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>469</v>
+        <v>553</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>470</v>
+        <v>554</v>
       </c>
     </row>
   </sheetData>

</xml_diff>